<commit_message>
feat(supplies): atualizar modelo excel para 3 colunas cod nome do material e cod prop
</commit_message>
<xml_diff>
--- a/docs/modelo_importacao_materiais.xlsx
+++ b/docs/modelo_importacao_materiais.xlsx
@@ -16,1098 +16,1644 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="364">
-  <si>
-    <t>CÓD.</t>
-  </si>
-  <si>
-    <t>DESCRIÇÃO</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="546">
+  <si>
+    <t>COD.</t>
+  </si>
+  <si>
+    <t>NOME DO MATERIAL</t>
+  </si>
+  <si>
+    <t>COD. PROP.</t>
   </si>
   <si>
     <t>1AB8</t>
   </si>
   <si>
-    <t xml:space="preserve">10GBASE-BXD SFP+ BiDi Tx1330/Rx1270nm 10km LC DDM</t>
+    <t>10GBASE-BXD SFP+ BiDi Tx1330/Rx1270nm 10km LC DDM</t>
+  </si>
+  <si>
+    <t>PRP-1AB8</t>
   </si>
   <si>
     <t>19E7</t>
   </si>
   <si>
-    <t xml:space="preserve">10GBASE-BXU SFP+ BiDi Tx1270/Rx1330nm 10KM LC DDM</t>
+    <t>10GBASE-BXU SFP+ BiDi Tx1270/Rx1330nm 10KM LC DDM</t>
+  </si>
+  <si>
+    <t>PRP-19E7</t>
   </si>
   <si>
     <t>6F24</t>
   </si>
   <si>
-    <t xml:space="preserve">40GBASE-LR4 QSFP+ 1310NM 10KM SMF LC DDM DUPLEX</t>
+    <t>40GBASE-LR4 QSFP+ 1310NM 10KM SMF LC DDM DUPLEX</t>
+  </si>
+  <si>
+    <t>PRP-6F24</t>
   </si>
   <si>
     <t>18ED</t>
   </si>
   <si>
-    <t xml:space="preserve">ABRAÇADEIRA BAP 3 DTC096 | 1200MM</t>
+    <t>ABRAÇADEIRA BAP 3 DTC096 | 1200MM</t>
+  </si>
+  <si>
+    <t>PRP-18ED</t>
   </si>
   <si>
     <t>6C7B</t>
   </si>
   <si>
-    <t xml:space="preserve">ABRAÇADEIRA BAP 4 DTC113 | 1000 MM</t>
+    <t>ABRAÇADEIRA BAP 4 DTC113 | 1000 MM</t>
+  </si>
+  <si>
+    <t>PRP-6C7B</t>
   </si>
   <si>
     <t>0D52</t>
   </si>
   <si>
-    <t xml:space="preserve">ABRACADEIRA NYLON | 10 CM PEQUENA DTC099</t>
+    <t>ABRACADEIRA NYLON | 10 CM PEQUENA DTC099</t>
+  </si>
+  <si>
+    <t>PRP-0D52</t>
   </si>
   <si>
     <t>267F</t>
   </si>
   <si>
-    <t xml:space="preserve">ABRAÇADEIRA NYLON | 20 CM MEDIA DTC099</t>
+    <t>ABRAÇADEIRA NYLON | 20 CM MEDIA DTC099</t>
+  </si>
+  <si>
+    <t>PRP-267F</t>
   </si>
   <si>
     <t>B961</t>
   </si>
   <si>
-    <t xml:space="preserve">ABRACADEIRA NYLON | 30 CM GRANDE DTC099</t>
+    <t>ABRACADEIRA NYLON | 30 CM GRANDE DTC099</t>
+  </si>
+  <si>
+    <t>PRP-B961</t>
   </si>
   <si>
     <t>279E</t>
   </si>
   <si>
-    <t xml:space="preserve">ADAPTADOR CONECTOR SC APC DTC146</t>
+    <t>ADAPTADOR CONECTOR SC APC DTC146</t>
+  </si>
+  <si>
+    <t>PRP-279E</t>
   </si>
   <si>
     <t>3FAD</t>
   </si>
   <si>
-    <t xml:space="preserve">ALÇA PREFORMADA | 10,8 A 11,7 MM</t>
+    <t>ALÇA PREFORMADA | 10,8 A 11,7 MM</t>
+  </si>
+  <si>
+    <t>PRP-3FAD</t>
   </si>
   <si>
     <t>A0F3</t>
   </si>
   <si>
-    <t xml:space="preserve">ALÇA PREFORMADA | 11,20 A 12,20 MM</t>
+    <t>ALÇA PREFORMADA | 11,20 A 12,20 MM</t>
+  </si>
+  <si>
+    <t>PRP-A0F3</t>
   </si>
   <si>
     <t>6CE9</t>
   </si>
   <si>
-    <t xml:space="preserve">ALÇA PREFORMADA | 4,8 A 5,3 MM DTC158</t>
+    <t>ALÇA PREFORMADA | 4,8 A 5,3 MM DTC158</t>
+  </si>
+  <si>
+    <t>PRP-6CE9</t>
   </si>
   <si>
     <t>C82F</t>
   </si>
   <si>
-    <t xml:space="preserve">ALÇA PREFORMADA | 6,8 a 7,4 MM</t>
+    <t>ALÇA PREFORMADA | 6,8 a 7,4 MM</t>
+  </si>
+  <si>
+    <t>PRP-C82F</t>
   </si>
   <si>
     <t>7A6C</t>
   </si>
   <si>
-    <t xml:space="preserve">ALCA PREFORMADA | 8,0 a 8,6 MM OPDE 1003</t>
+    <t>ALCA PREFORMADA | 8,0 a 8,6 MM OPDE 1003</t>
+  </si>
+  <si>
+    <t>PRP-7A6C</t>
   </si>
   <si>
     <t>2BFC</t>
   </si>
   <si>
-    <t xml:space="preserve">ALÇA PREFORMADA | 9,6 A 10,6 MM OPDE 1021</t>
+    <t>ALÇA PREFORMADA | 9,6 A 10,6 MM OPDE 1021</t>
+  </si>
+  <si>
+    <t>PRP-2BFC</t>
   </si>
   <si>
     <t>70F3</t>
   </si>
   <si>
-    <t xml:space="preserve">ALCA PREFORMADA OPDE 1002 12,4 A 13,4MM</t>
+    <t>ALCA PREFORMADA OPDE 1002 12,4 A 13,4MM</t>
+  </si>
+  <si>
+    <t>PRP-70F3</t>
   </si>
   <si>
     <t>F89E</t>
   </si>
   <si>
-    <t xml:space="preserve">ALÇA PREFORMADA OPDE 1032 9,6 A 10,6MM DTC309</t>
+    <t>ALÇA PREFORMADA OPDE 1032 9,6 A 10,6MM DTC309</t>
+  </si>
+  <si>
+    <t>PRP-F89E</t>
   </si>
   <si>
     <t>B6CA</t>
   </si>
   <si>
-    <t xml:space="preserve">ALÇA PREFORMADA P/ CORDOALHA DIELÉTRICA | 6,4 MM</t>
+    <t>ALÇA PREFORMADA P/ CORDOALHA DIELÉTRICA | 6,4 MM</t>
+  </si>
+  <si>
+    <t>PRP-B6CA</t>
   </si>
   <si>
     <t>4618</t>
   </si>
   <si>
-    <t xml:space="preserve">ALCOOL ISOPROPILICO DTCO97</t>
+    <t>ALCOOL ISOPROPILICO DTCO97</t>
+  </si>
+  <si>
+    <t>PRP-4618</t>
   </si>
   <si>
     <t>741F</t>
   </si>
   <si>
-    <t xml:space="preserve">ANEL AGUIA AGF DTC133</t>
+    <t>ANEL AGUIA AGF DTC133</t>
+  </si>
+  <si>
+    <t>PRP-741F</t>
   </si>
   <si>
     <t>D45C</t>
   </si>
   <si>
-    <t xml:space="preserve">ANTENA NANO STATION 5 UBIQUITI</t>
+    <t>ANTENA NANO STATION 5 UBIQUITI</t>
+  </si>
+  <si>
+    <t>PRP-D45C</t>
   </si>
   <si>
     <t>AC47</t>
   </si>
   <si>
-    <t xml:space="preserve">BANDEJA FIXA P/RACK</t>
+    <t>BANDEJA FIXA P/RACK</t>
+  </si>
+  <si>
+    <t>PRP-AC47</t>
   </si>
   <si>
     <t>324A</t>
   </si>
   <si>
-    <t xml:space="preserve">BANDEJA FIXA RACK 1U 700MM</t>
+    <t>BANDEJA FIXA RACK 1U 700MM</t>
+  </si>
+  <si>
+    <t>PRP-324A</t>
   </si>
   <si>
     <t>428E</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO CORDOALHA DIELETRICA 4,8MM</t>
+    <t>CABO CORDOALHA DIELETRICA 4,8MM</t>
+  </si>
+  <si>
+    <t>PRP-428E</t>
   </si>
   <si>
     <t>D154</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO CORDOALHA DIELETRICA 6,4MM DTCI32</t>
+    <t>CABO CORDOALHA DIELETRICA 6,4MM DTCI32</t>
+  </si>
+  <si>
+    <t>PRP-D154</t>
   </si>
   <si>
     <t>ECFA</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO DE REDE UTP CAT5E DTC141</t>
+    <t>CABO DE REDE UTP CAT5E DTC141</t>
+  </si>
+  <si>
+    <t>PRP-ECFA</t>
   </si>
   <si>
     <t>FD2C</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO ENERGIA MERAKI MT80 BR</t>
+    <t>CABO ENERGIA MERAKI MT80 BR</t>
+  </si>
+  <si>
+    <t>PRP-FD2C</t>
   </si>
   <si>
     <t>E8DA</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO FIBRA OPTICA AS-80 MINI 06FO (CFOA)</t>
+    <t>CABO FIBRA OPTICA AS-80 MINI 06FO (CFOA)</t>
+  </si>
+  <si>
+    <t>PRP-E8DA</t>
   </si>
   <si>
     <t>3D4F</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO FIBRA OPTICA AS-80 TS 72FO (CFOA) DTC 062</t>
+    <t>CABO FIBRA OPTICA AS-80 TS 72FO (CFOA) DTC 062</t>
+  </si>
+  <si>
+    <t>PRP-3D4F</t>
   </si>
   <si>
     <t>C20B</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO FIBRA OPTICA ASU-80 12FO (CFOA) DTC 060</t>
+    <t>CABO FIBRA OPTICA ASU-80 12FO (CFOA) DTC 060</t>
+  </si>
+  <si>
+    <t>PRP-C20B</t>
   </si>
   <si>
     <t>B2D5</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO FLEX AZUL1KV 10MM</t>
+    <t>CABO FLEX AZUL1KV 10MM</t>
+  </si>
+  <si>
+    <t>PRP-B2D5</t>
   </si>
   <si>
     <t>58FC</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO FLEX PRETO 1KV 10MM</t>
+    <t>CABO FLEX PRETO 1KV 10MM</t>
+  </si>
+  <si>
+    <t>PRP-58FC</t>
   </si>
   <si>
     <t>57EF</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO FLEX VERDE 1KV 10MM</t>
+    <t>CABO FLEX VERDE 1KV 10MM</t>
+  </si>
+  <si>
+    <t>PRP-57EF</t>
   </si>
   <si>
     <t>72A3</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO MPO FEMEA 12F OM4 50/125 TIPO B LSZH 5M</t>
+    <t>CABO MPO FEMEA 12F OM4 50/125 TIPO B LSZH 5M</t>
+  </si>
+  <si>
+    <t>PRP-72A3</t>
   </si>
   <si>
     <t>F241</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO OPTICO AS120 12 FO DTC207</t>
+    <t>CABO OPTICO AS120 12 FO DTC207</t>
+  </si>
+  <si>
+    <t>PRP-F241</t>
   </si>
   <si>
     <t>269C</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO OPTICO AS80 36FO</t>
+    <t>CABO OPTICO AS80 36FO</t>
+  </si>
+  <si>
+    <t>PRP-269C</t>
   </si>
   <si>
     <t>A14C</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO OPTICO CFOA-SM-AS80-S 48F TS</t>
+    <t>CABO OPTICO CFOA-SM-AS80-S 48F TS</t>
+  </si>
+  <si>
+    <t>PRP-A14C</t>
   </si>
   <si>
     <t>32E5</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO OPTICO CIRCULAR AS80 4FO DTC063</t>
+    <t>CABO OPTICO CIRCULAR AS80 4FO DTC063</t>
+  </si>
+  <si>
+    <t>PRP-32E5</t>
   </si>
   <si>
     <t>A03F</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO OPTICO TS AS200 12FO</t>
+    <t>CABO OPTICO TS AS200 12FO</t>
+  </si>
+  <si>
+    <t>PRP-A03F</t>
   </si>
   <si>
     <t>2CA8</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO OPTICO TS AS200 24FO</t>
+    <t>CABO OPTICO TS AS200 24FO</t>
+  </si>
+  <si>
+    <t>PRP-2CA8</t>
   </si>
   <si>
     <t>ECB7</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO OPTICO TS AS80 24FO DTC207</t>
+    <t>CABO OPTICO TS AS80 24FO DTC207</t>
+  </si>
+  <si>
+    <t>PRP-ECB7</t>
   </si>
   <si>
     <t>7AC1</t>
   </si>
   <si>
-    <t xml:space="preserve">CAIXA DE EMENDA OPTICA TRONCAL E LR 36FO DPR (CEO) - DTC 041</t>
+    <t>CAIXA DE EMENDA OPTICA TRONCAL E LR 36FO DPR (CEO) - DTC 041</t>
+  </si>
+  <si>
+    <t>PRP-7AC1</t>
   </si>
   <si>
     <t>650B</t>
   </si>
   <si>
-    <t xml:space="preserve">CAIXA DE TRANSIÇÃO FTTA 12FO DTC131 (TERMINADO OPTICO)</t>
+    <t>CAIXA DE TRANSIÇÃO FTTA 12FO DTC131 (TERMINADO OPTICO)</t>
+  </si>
+  <si>
+    <t>PRP-650B</t>
   </si>
   <si>
     <t>D9FE</t>
   </si>
   <si>
-    <t xml:space="preserve">CAIXA EMENDA OPTICA 24 FO</t>
+    <t>CAIXA EMENDA OPTICA 24 FO</t>
+  </si>
+  <si>
+    <t>PRP-D9FE</t>
   </si>
   <si>
     <t>4B9D</t>
   </si>
   <si>
-    <t xml:space="preserve">CAIXA HERMETICA OUTDOOR 35X35X35CM</t>
+    <t>CAIXA HERMETICA OUTDOOR 35X35X35CM</t>
+  </si>
+  <si>
+    <t>PRP-4B9D</t>
   </si>
   <si>
     <t>B549</t>
   </si>
   <si>
-    <t xml:space="preserve">CAMERA FIXA DH HFW 5241 EN ZE</t>
+    <t>CAMERA FIXA DH HFW 5241 EN ZE</t>
+  </si>
+  <si>
+    <t>PRP-B549</t>
   </si>
   <si>
     <t>C935</t>
   </si>
   <si>
-    <t xml:space="preserve">CHAPA M 14MM - SUPORTE REFORÇADO P/ BAP</t>
+    <t>CHAPA M 14MM - SUPORTE REFORÇADO P/ BAP</t>
+  </si>
+  <si>
+    <t>PRP-C935</t>
   </si>
   <si>
     <t>4D3A</t>
   </si>
   <si>
-    <t xml:space="preserve">CÍSCO FIREWALL MERAKI MX68</t>
+    <t>CÍSCO FIREWALL MERAKI MX68</t>
+  </si>
+  <si>
+    <t>PRP-4D3A</t>
   </si>
   <si>
     <t>0CB7</t>
   </si>
   <si>
-    <t xml:space="preserve">CONECTOR MECANICO DE CAMPO SC-APC VERDE - DTC 042</t>
+    <t>CONECTOR MECANICO DE CAMPO SC-APC VERDE - DTC 042</t>
+  </si>
+  <si>
+    <t>PRP-0CB7</t>
   </si>
   <si>
     <t>FB32</t>
   </si>
   <si>
-    <t xml:space="preserve">CONECTOR MECANICO DE CAMPO SC-UPC AZUL - DTC 043</t>
+    <t>CONECTOR MECANICO DE CAMPO SC-UPC AZUL - DTC 043</t>
+  </si>
+  <si>
+    <t>PRP-FB32</t>
   </si>
   <si>
     <t>32E7</t>
   </si>
   <si>
-    <t xml:space="preserve">CONECTOR RJ45</t>
+    <t>CONECTOR RJ45</t>
+  </si>
+  <si>
+    <t>PRP-32E7</t>
   </si>
   <si>
     <t>CFED</t>
   </si>
   <si>
-    <t xml:space="preserve">CONVERSOR MIDIA CTS 600 EF LXA GIGABIT</t>
+    <t>CONVERSOR MIDIA CTS 600 EF LXA GIGABIT</t>
+  </si>
+  <si>
+    <t>PRP-CFED</t>
   </si>
   <si>
     <t>B708</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDAO OPTICO DUPLEX SM LC UPC LC UPC 15M DTC143</t>
+    <t>CORDAO OPTICO DUPLEX SM LC UPC LC UPC 15M DTC143</t>
+  </si>
+  <si>
+    <t>PRP-B708</t>
   </si>
   <si>
     <t>E319</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDÃO OPTICO DUPLEX SM LC UPC LC UPC 30M</t>
+    <t>CORDÃO OPTICO DUPLEX SM LC UPC LC UPC 30M</t>
+  </si>
+  <si>
+    <t>PRP-E319</t>
   </si>
   <si>
     <t>F293</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDÃO OPTICO DUPLEX SM SC APC LC APC 3M DTC143</t>
+    <t>CORDÃO OPTICO DUPLEX SM SC APC LC APC 3M DTC143</t>
+  </si>
+  <si>
+    <t>PRP-F293</t>
   </si>
   <si>
     <t>4F5D</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDAO OPTICO DUPLEX SM SC APC LC UPC 2,5M</t>
+    <t>CORDAO OPTICO DUPLEX SM SC APC LC UPC 2,5M</t>
+  </si>
+  <si>
+    <t>PRP-4F5D</t>
   </si>
   <si>
     <t>B389</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDÃO OPTICO DUPLEX SM SC APC LC UPC 5M DTC143</t>
+    <t>CORDÃO OPTICO DUPLEX SM SC APC LC UPC 5M DTC143</t>
+  </si>
+  <si>
+    <t>PRP-B389</t>
   </si>
   <si>
     <t>BD35</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDAO OPTICO DUPLEX SM SC APC LC UPC 7M</t>
+    <t>CORDAO OPTICO DUPLEX SM SC APC LC UPC 7M</t>
+  </si>
+  <si>
+    <t>PRP-BD35</t>
   </si>
   <si>
     <t>D78A</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDÃO OPTICO DUPLEX SM SC APC LC UPT 10M</t>
+    <t>CORDÃO OPTICO DUPLEX SM SC APC LC UPT 10M</t>
+  </si>
+  <si>
+    <t>PRP-D78A</t>
   </si>
   <si>
     <t>8FEC</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDAO OPTICO DUPLEX-SM LC-PC/ LC-PC 5M</t>
+    <t>CORDAO OPTICO DUPLEX-SM LC-PC/ LC-PC 5M</t>
+  </si>
+  <si>
+    <t>PRP-8FEC</t>
   </si>
   <si>
     <t>C704</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDAO OPTICO PIGTAIL SIMPLEX  SC UPC (APC)</t>
+    <t>CORDAO OPTICO PIGTAIL SIMPLEX  SC UPC (APC)</t>
+  </si>
+  <si>
+    <t>PRP-C704</t>
   </si>
   <si>
     <t>A481</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDÃO OPTICO PIGTAIL SIMPLEX SC APC</t>
+    <t>CORDÃO OPTICO PIGTAIL SIMPLEX SC APC</t>
+  </si>
+  <si>
+    <t>PRP-A481</t>
   </si>
   <si>
     <t>EFCA</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDÃO OPTICO SIMPLEX SC APC LC APC 5M DTC143</t>
+    <t>CORDÃO OPTICO SIMPLEX SC APC LC APC 5M DTC143</t>
+  </si>
+  <si>
+    <t>PRP-EFCA</t>
   </si>
   <si>
     <t>F4EA</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDAO OPTICO SIMPLEX SM LC APC LC APC 3M DTC143</t>
+    <t>CORDAO OPTICO SIMPLEX SM LC APC LC APC 3M DTC143</t>
+  </si>
+  <si>
+    <t>PRP-F4EA</t>
   </si>
   <si>
     <t>1A67</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDÃO OPTICO SIMPLEX SM LC APC SC APC 2,5M</t>
+    <t>CORDÃO OPTICO SIMPLEX SM LC APC SC APC 2,5M</t>
+  </si>
+  <si>
+    <t>PRP-1A67</t>
   </si>
   <si>
     <t>01EC</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDAO OPTICO SIMPLEX SM LC PC SC APC  2,5M</t>
+    <t>CORDAO OPTICO SIMPLEX SM LC PC SC APC  2,5M</t>
+  </si>
+  <si>
+    <t>PRP-01EC</t>
   </si>
   <si>
     <t>32ED</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDAO OPTICO SIMPLEX SM LC-UPC/SC-APC 2,5M</t>
+    <t>CORDAO OPTICO SIMPLEX SM LC-UPC/SC-APC 2,5M</t>
+  </si>
+  <si>
+    <t>PRP-32ED</t>
   </si>
   <si>
     <t>91C2</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDÃO OPTICO SIMPLEX SM SC APC LC APC 10M DTC143</t>
+    <t>CORDÃO OPTICO SIMPLEX SM SC APC LC APC 10M DTC143</t>
+  </si>
+  <si>
+    <t>PRP-91C2</t>
   </si>
   <si>
     <t>2DB3</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDÃO OPTICO SIMPLEX SM SC APC LC APC 3M DTC143</t>
+    <t>CORDÃO OPTICO SIMPLEX SM SC APC LC APC 3M DTC143</t>
+  </si>
+  <si>
+    <t>PRP-2DB3</t>
   </si>
   <si>
     <t>C81E</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDAO OPTICO SIMPLEX SM SC APC LC UPC 3M DTC I43</t>
+    <t>CORDAO OPTICO SIMPLEX SM SC APC LC UPC 3M DTC I43</t>
+  </si>
+  <si>
+    <t>PRP-C81E</t>
   </si>
   <si>
     <t>A602</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDÃO OPTICO SIMPLEX SM SC APC LC UPC 5MT SM DTC143</t>
+    <t>CORDÃO OPTICO SIMPLEX SM SC APC LC UPC 5MT SM DTC143</t>
+  </si>
+  <si>
+    <t>PRP-A602</t>
   </si>
   <si>
     <t>A145</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDAO OPTICO SIMPLEX SM SC APC SC APC 2,5M</t>
+    <t>CORDAO OPTICO SIMPLEX SM SC APC SC APC 2,5M</t>
+  </si>
+  <si>
+    <t>PRP-A145</t>
   </si>
   <si>
     <t>385B</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDÃO OPTICO SIMPLEX SM SC APC SC APC 2MT</t>
+    <t>CORDÃO OPTICO SIMPLEX SM SC APC SC APC 2MT</t>
+  </si>
+  <si>
+    <t>PRP-385B</t>
   </si>
   <si>
     <t>4FAB</t>
   </si>
   <si>
-    <t xml:space="preserve">CORDAO OPTICO SIMPLEX SM SC/APC LC/APC 20M DTC143</t>
+    <t>CORDAO OPTICO SIMPLEX SM SC/APC LC/APC 20M DTC143</t>
+  </si>
+  <si>
+    <t>PRP-4FAB</t>
   </si>
   <si>
     <t>FB03</t>
   </si>
   <si>
-    <t xml:space="preserve">DIO PADRÃO 19 SM C/PIGTAIL SC/APC 12FO</t>
+    <t>DIO PADRÃO 19 SM C/PIGTAIL SC/APC 12FO</t>
+  </si>
+  <si>
+    <t>PRP-FB03</t>
   </si>
   <si>
     <t>5FD6</t>
   </si>
   <si>
-    <t xml:space="preserve">DIO PADRAO 19 SM C/PIGTAIL SC/APC 24FO</t>
+    <t>DIO PADRAO 19 SM C/PIGTAIL SC/APC 24FO</t>
+  </si>
+  <si>
+    <t>PRP-5FD6</t>
   </si>
   <si>
     <t>2B7F</t>
   </si>
   <si>
-    <t xml:space="preserve">DIO PADRAO 19 SM C/PIGTAIL SC/APC 72FO</t>
+    <t>DIO PADRAO 19 SM C/PIGTAIL SC/APC 72FO</t>
+  </si>
+  <si>
+    <t>PRP-2B7F</t>
   </si>
   <si>
     <t>07F5</t>
   </si>
   <si>
-    <t xml:space="preserve">DISJUNTOR TRIPOLAR CURVA C 100A</t>
+    <t>DISJUNTOR TRIPOLAR CURVA C 100A</t>
+  </si>
+  <si>
+    <t>PRP-07F5</t>
   </si>
   <si>
     <t>86A5</t>
   </si>
   <si>
-    <t xml:space="preserve">DISJUNTOR TRIPOLAR CURVA C 40A</t>
+    <t>DISJUNTOR TRIPOLAR CURVA C 40A</t>
+  </si>
+  <si>
+    <t>PRP-86A5</t>
   </si>
   <si>
     <t>3F2B</t>
   </si>
   <si>
-    <t xml:space="preserve">DISJUNTOR TRIPOLAR CURVA C 63A</t>
+    <t>DISJUNTOR TRIPOLAR CURVA C 63A</t>
+  </si>
+  <si>
+    <t>PRP-3F2B</t>
   </si>
   <si>
     <t>264C</t>
   </si>
   <si>
-    <t xml:space="preserve">DISJUNTOR TRIPOLAR CURVA C 80A</t>
+    <t>DISJUNTOR TRIPOLAR CURVA C 80A</t>
+  </si>
+  <si>
+    <t>PRP-264C</t>
   </si>
   <si>
     <t>F730</t>
   </si>
   <si>
-    <t xml:space="preserve">DISJUNTOR UNIPOLAR CURVA C 10A</t>
+    <t>DISJUNTOR UNIPOLAR CURVA C 10A</t>
+  </si>
+  <si>
+    <t>PRP-F730</t>
   </si>
   <si>
     <t>D267</t>
   </si>
   <si>
-    <t xml:space="preserve">DISJUNTOR UNIPOLAR CURVA C 20A</t>
+    <t>DISJUNTOR UNIPOLAR CURVA C 20A</t>
+  </si>
+  <si>
+    <t>PRP-D267</t>
   </si>
   <si>
     <t>E028</t>
   </si>
   <si>
-    <t xml:space="preserve">DISJUNTOR UNIPOLAR CURVA C 25A</t>
+    <t>DISJUNTOR UNIPOLAR CURVA C 25A</t>
+  </si>
+  <si>
+    <t>PRP-E028</t>
   </si>
   <si>
     <t>F2E8</t>
   </si>
   <si>
-    <t xml:space="preserve">DISJUNTOR UNIPOLAR CURVA C 32A</t>
+    <t>DISJUNTOR UNIPOLAR CURVA C 32A</t>
+  </si>
+  <si>
+    <t>PRP-F2E8</t>
   </si>
   <si>
     <t>BC4A</t>
   </si>
   <si>
-    <t xml:space="preserve">DISJUNTOR UNIPOLAR CURVA C 50A</t>
+    <t>DISJUNTOR UNIPOLAR CURVA C 50A</t>
+  </si>
+  <si>
+    <t>PRP-BC4A</t>
   </si>
   <si>
     <t>DFEB</t>
   </si>
   <si>
-    <t xml:space="preserve">DMSWITCH 2104G EDD DATACOM 2E1</t>
+    <t>DMSWITCH 2104G EDD DATACOM 2E1</t>
+  </si>
+  <si>
+    <t>PRP-DFEB</t>
   </si>
   <si>
     <t>17CF</t>
   </si>
   <si>
-    <t xml:space="preserve">DROP COMPACTO LOW FRICTION MARRON 01FO - DTC 204</t>
+    <t>DROP COMPACTO LOW FRICTION MARRON 01FO - DTC 204</t>
+  </si>
+  <si>
+    <t>PRP-17CF</t>
   </si>
   <si>
     <t>3AEB</t>
   </si>
   <si>
-    <t xml:space="preserve">ESPIRAL TUBE PLASTICO 1/4 DTC248</t>
+    <t>ESPIRAL TUBE PLASTICO 1/4 DTC248</t>
+  </si>
+  <si>
+    <t>PRP-3AEB</t>
   </si>
   <si>
     <t>9F5A</t>
   </si>
   <si>
-    <t xml:space="preserve">ESTICADOR DROP CUNHA ANEL AGEF DTC135</t>
+    <t>ESTICADOR DROP CUNHA ANEL AGEF DTC135</t>
+  </si>
+  <si>
+    <t>PRP-9F5A</t>
   </si>
   <si>
     <t>9B76</t>
   </si>
   <si>
-    <t xml:space="preserve">ESTICADOR DROP CUNHA ROLDANA DTC243</t>
+    <t>ESTICADOR DROP CUNHA ROLDANA DTC243</t>
+  </si>
+  <si>
+    <t>PRP-9B76</t>
   </si>
   <si>
     <t>E3C6</t>
   </si>
   <si>
-    <t xml:space="preserve">EXTENSAO OPTICA SC APC 15M ALTA POTENCIA</t>
+    <t>EXTENSAO OPTICA SC APC 15M ALTA POTENCIA</t>
+  </si>
+  <si>
+    <t>PRP-E3C6</t>
   </si>
   <si>
     <t>C467</t>
   </si>
   <si>
-    <t xml:space="preserve">EXTENSÃO OPTICO SIMPLEX SM SC UPC 3M DTC143</t>
+    <t>EXTENSÃO OPTICO SIMPLEX SM SC UPC 3M DTC143</t>
+  </si>
+  <si>
+    <t>PRP-C467</t>
   </si>
   <si>
     <t>1CBA</t>
   </si>
   <si>
-    <t xml:space="preserve">FECHO DE AÇO INOXIDAVEL - DTC 134</t>
+    <t>FECHO DE AÇO INOXIDAVEL - DTC 134</t>
+  </si>
+  <si>
+    <t>PRP-1CBA</t>
   </si>
   <si>
     <t>AE39</t>
   </si>
   <si>
-    <t xml:space="preserve">FIO DE ESPINAR DIELÉTRICO DTC130</t>
+    <t>FIO DE ESPINAR DIELÉTRICO DTC130</t>
+  </si>
+  <si>
+    <t>PRP-AE39</t>
   </si>
   <si>
     <t>2610</t>
   </si>
   <si>
-    <t xml:space="preserve">FIO DE ESPINAR ISOLADO - DTC 131</t>
+    <t>FIO DE ESPINAR ISOLADO - DTC 131</t>
+  </si>
+  <si>
+    <t>PRP-2610</t>
   </si>
   <si>
     <t>B195</t>
   </si>
   <si>
-    <t xml:space="preserve">FIREWALL FORTGATE 200F</t>
+    <t>FIREWALL FORTGATE 200F</t>
+  </si>
+  <si>
+    <t>PRP-B195</t>
   </si>
   <si>
     <t>9524</t>
   </si>
   <si>
-    <t xml:space="preserve">FIREWALL FORTGATE 40F</t>
+    <t>FIREWALL FORTGATE 40F</t>
+  </si>
+  <si>
+    <t>PRP-9524</t>
   </si>
   <si>
     <t>6723</t>
   </si>
   <si>
-    <t xml:space="preserve">FIREWALL FORTGATE 60F</t>
+    <t>FIREWALL FORTGATE 60F</t>
+  </si>
+  <si>
+    <t>PRP-6723</t>
   </si>
   <si>
     <t>6E49</t>
   </si>
   <si>
-    <t xml:space="preserve">FIREWALL FORTGATE 100F</t>
+    <t>FIREWALL FORTGATE 100F</t>
+  </si>
+  <si>
+    <t>PRP-6E49</t>
   </si>
   <si>
     <t>B239</t>
   </si>
   <si>
-    <t xml:space="preserve">FITA AÇO INOXIDAVEL LITORAL DTC134</t>
+    <t>FITA AÇO INOXIDAVEL LITORAL DTC134</t>
+  </si>
+  <si>
+    <t>PRP-B239</t>
   </si>
   <si>
     <t>A395</t>
   </si>
   <si>
-    <t xml:space="preserve">FITA DE AUTO FUSAO DTC106</t>
+    <t>FITA DE AUTO FUSAO DTC106</t>
+  </si>
+  <si>
+    <t>PRP-A395</t>
   </si>
   <si>
     <t>A35B</t>
   </si>
   <si>
-    <t xml:space="preserve">FITA ISOLANTE DE PVC - DTC 107</t>
+    <t>FITA ISOLANTE DE PVC - DTC 107</t>
+  </si>
+  <si>
+    <t>PRP-A35B</t>
   </si>
   <si>
     <t>530D</t>
   </si>
   <si>
-    <t xml:space="preserve">FIXADOR INTERNO DE CABOS METALICOS/UTP MOD-M - DTC 064</t>
+    <t>FIXADOR INTERNO DE CABOS METALICOS/UTP MOD-M - DTC 064</t>
+  </si>
+  <si>
+    <t>PRP-530D</t>
   </si>
   <si>
     <t>37ED</t>
   </si>
   <si>
-    <t xml:space="preserve">FONTE ALIMENTAÇÃO POE 24V 1A</t>
+    <t>FONTE ALIMENTAÇÃO POE 24V 1A</t>
+  </si>
+  <si>
+    <t>PRP-37ED</t>
   </si>
   <si>
     <t>7F28</t>
   </si>
   <si>
-    <t xml:space="preserve">FONTE NOBREAK 24V/7A VOLT</t>
+    <t>FONTE NOBREAK 24V/7A VOLT</t>
+  </si>
+  <si>
+    <t>PRP-7F28</t>
   </si>
   <si>
     <t>652E</t>
   </si>
   <si>
-    <t xml:space="preserve">FONTE POE 24V</t>
+    <t>FONTE POE 24V</t>
+  </si>
+  <si>
+    <t>PRP-652E</t>
   </si>
   <si>
     <t>8F72</t>
   </si>
   <si>
-    <t xml:space="preserve">FONTE RETIFICADORA HUAWEI S6730 DC POWER 1000W</t>
+    <t>FONTE RETIFICADORA HUAWEI S6730 DC POWER 1000W</t>
+  </si>
+  <si>
+    <t>PRP-8F72</t>
   </si>
   <si>
     <t>8E15</t>
   </si>
   <si>
-    <t xml:space="preserve">GBIC QSFP28 SR4 LIGHTPAD i6400G 100G</t>
+    <t>GBIC QSFP28 SR4 LIGHTPAD i6400G 100G</t>
+  </si>
+  <si>
+    <t>PRP-8E15</t>
   </si>
   <si>
     <t>CE32</t>
   </si>
   <si>
-    <t xml:space="preserve">GBIC SFP 1.25G 10KM LC DUPLEX FREQ. 1310</t>
+    <t>GBIC SFP 1.25G 10KM LC DUPLEX FREQ. 1310</t>
+  </si>
+  <si>
+    <t>PRP-CE32</t>
   </si>
   <si>
     <t>051D</t>
   </si>
   <si>
-    <t xml:space="preserve">LAÇO PREFORMADO CT 155 6,5 A 7,5MM</t>
+    <t>LAÇO PREFORMADO CT 155 6,5 A 7,5MM</t>
+  </si>
+  <si>
+    <t>PRP-051D</t>
   </si>
   <si>
     <t>72D0</t>
   </si>
   <si>
-    <t xml:space="preserve">LACO PREFORMADO СТ 1561 11.2 A 12.2MM</t>
+    <t>LACO PREFORMADO СТ 1561 11.2 A 12.2MM</t>
+  </si>
+  <si>
+    <t>PRP-72D0</t>
   </si>
   <si>
     <t>5A40</t>
   </si>
   <si>
-    <t xml:space="preserve">MINI CAIXA EMENDA PREDIAL 12FO LINEAR DTC244</t>
+    <t>MINI CAIXA EMENDA PREDIAL 12FO LINEAR DTC244</t>
+  </si>
+  <si>
+    <t>PRP-5A40</t>
   </si>
   <si>
     <t>DAE8</t>
   </si>
   <si>
-    <t xml:space="preserve">MINI CAIXA EMENDA PREDIAL 12FO TOPO DTC244</t>
+    <t>MINI CAIXA EMENDA PREDIAL 12FO TOPO DTC244</t>
+  </si>
+  <si>
+    <t>PRP-DAE8</t>
   </si>
   <si>
     <t>3F74</t>
   </si>
   <si>
-    <t xml:space="preserve">MODULO QSFP + LR4 1310NM 40G 20KM</t>
+    <t>MODULO QSFP + LR4 1310NM 40G 20KM</t>
+  </si>
+  <si>
+    <t>PRP-3F74</t>
   </si>
   <si>
     <t>0EA3</t>
   </si>
   <si>
-    <t xml:space="preserve">MODULO QSFP28 LR4 1310NM 100G 20KM</t>
+    <t>MODULO QSFP28 LR4 1310NM 100G 20KM</t>
+  </si>
+  <si>
+    <t>PRP-0EA3</t>
   </si>
   <si>
     <t>E6A0</t>
   </si>
   <si>
-    <t xml:space="preserve">MODULO QSFP28 SR4 850NM 100G 100M DTC304</t>
+    <t>MODULO QSFP28 SR4 850NM 100G 100M DTC304</t>
+  </si>
+  <si>
+    <t>PRP-E6A0</t>
   </si>
   <si>
     <t>5804</t>
   </si>
   <si>
-    <t xml:space="preserve">MODULO SFP BIDI 1310NM 1550NM 1.25G 10 KM</t>
+    <t>MODULO SFP BIDI 1310NM 1550NM 1.25G 10 KM</t>
+  </si>
+  <si>
+    <t>PRP-5804</t>
   </si>
   <si>
     <t>A16F</t>
   </si>
   <si>
-    <t xml:space="preserve">MODULO SFP RJ45 1.25G 100M DTC312</t>
+    <t>MODULO SFP RJ45 1.25G 100M DTC312</t>
+  </si>
+  <si>
+    <t>PRP-A16F</t>
   </si>
   <si>
     <t>5027</t>
   </si>
   <si>
-    <t xml:space="preserve">MODULO SFP+ BIDI 1270NM 1330NM 10G 40KM</t>
+    <t>MODULO SFP+ BIDI 1270NM 1330NM 10G 40KM</t>
+  </si>
+  <si>
+    <t>PRP-5027</t>
   </si>
   <si>
     <t>EF2D</t>
   </si>
   <si>
-    <t xml:space="preserve">MODULO SFP+ BIDI 1330NM 1270NM 10G 20KM</t>
+    <t>MODULO SFP+ BIDI 1330NM 1270NM 10G 20KM</t>
+  </si>
+  <si>
+    <t>PRP-EF2D</t>
   </si>
   <si>
     <t>3FBC</t>
   </si>
   <si>
-    <t xml:space="preserve">MODULO SFP+ SR 850NM 10G 300M DTC234</t>
+    <t>MODULO SFP+ SR 850NM 10G 300M DTC234</t>
+  </si>
+  <si>
+    <t>PRP-3FBC</t>
   </si>
   <si>
     <t>8915</t>
   </si>
   <si>
-    <t xml:space="preserve">MODULO SFP+BIDI 1330NM 1270NM 10G 40KM</t>
+    <t>MODULO SFP+BIDI 1330NM 1270NM 10G 40KM</t>
+  </si>
+  <si>
+    <t>PRP-8915</t>
   </si>
   <si>
     <t>D7F0</t>
   </si>
   <si>
-    <t xml:space="preserve">ONT G420W FURUKAWA WIFI 6</t>
+    <t>ONT G420W FURUKAWA WIFI 6</t>
+  </si>
+  <si>
+    <t>PRP-D7F0</t>
   </si>
   <si>
     <t>318D</t>
   </si>
   <si>
-    <t xml:space="preserve">ONT GPON HG8010H BRIDGE 1PORTA-HUAWEI</t>
+    <t>ONT GPON HG8010H BRIDGE 1PORTA-HUAWEI</t>
+  </si>
+  <si>
+    <t>PRP-318D</t>
   </si>
   <si>
     <t>F409</t>
   </si>
   <si>
-    <t xml:space="preserve">ONU BRIDGE FURUKAWA</t>
+    <t>ONU BRIDGE FURUKAWA</t>
+  </si>
+  <si>
+    <t>PRP-F409</t>
   </si>
   <si>
     <t>FB0A</t>
   </si>
   <si>
-    <t xml:space="preserve">ONU BRIDGE HUAWEI</t>
+    <t>ONU BRIDGE HUAWEI</t>
+  </si>
+  <si>
+    <t>PRP-FB0A</t>
   </si>
   <si>
     <t>D65C</t>
   </si>
   <si>
-    <t xml:space="preserve">ONU FURUKAWA 2.4 GHZ</t>
+    <t>ONU FURUKAWA 2.4 GHZ</t>
+  </si>
+  <si>
+    <t>PRP-D65C</t>
   </si>
   <si>
     <t>7451</t>
   </si>
   <si>
-    <t xml:space="preserve">ONU HUAWEI 2.4GHZ</t>
+    <t>ONU HUAWEI 2.4GHZ</t>
+  </si>
+  <si>
+    <t>PRP-7451</t>
   </si>
   <si>
     <t>0FB7</t>
   </si>
   <si>
-    <t xml:space="preserve">ONU HUAWEI 5.0GHz</t>
+    <t>ONU HUAWEI 5.0GHz</t>
+  </si>
+  <si>
+    <t>PRP-0FB7</t>
   </si>
   <si>
     <t>BAC1</t>
   </si>
   <si>
-    <t xml:space="preserve">PAINEL DISJUNTORES 20POSIÇÕES</t>
+    <t>PAINEL DISJUNTORES 20POSIÇÕES</t>
+  </si>
+  <si>
+    <t>PRP-BAC1</t>
   </si>
   <si>
     <t>A6D2</t>
   </si>
   <si>
-    <t xml:space="preserve">PARAFUSO FRANCES C/PORCA</t>
+    <t>PARAFUSO FRANCES C/PORCA</t>
+  </si>
+  <si>
+    <t>PRP-A6D2</t>
   </si>
   <si>
     <t>C4DA</t>
   </si>
   <si>
-    <t xml:space="preserve">PARAFUSO PITAO DTC 013</t>
+    <t>PARAFUSO PITAO DTC 013</t>
+  </si>
+  <si>
+    <t>PRP-C4DA</t>
   </si>
   <si>
     <t>52D6</t>
   </si>
   <si>
-    <t xml:space="preserve">PATCH CORD CAT5 1,5MT</t>
+    <t>PATCH CORD CAT5 1,5MT</t>
+  </si>
+  <si>
+    <t>PRP-52D6</t>
   </si>
   <si>
     <t>BE0A</t>
   </si>
   <si>
-    <t xml:space="preserve">PIGTAIL OPTICO SIMPLEX SM LC UPC 1,5M DTC140</t>
+    <t>PIGTAIL OPTICO SIMPLEX SM LC UPC 1,5M DTC140</t>
+  </si>
+  <si>
+    <t>PRP-BE0A</t>
   </si>
   <si>
     <t>4D57</t>
   </si>
   <si>
-    <t xml:space="preserve">PIGTAIL OPTICO SIMPLEX SM SC UPC 2,5M</t>
+    <t>PIGTAIL OPTICO SIMPLEX SM SC UPC 2,5M</t>
+  </si>
+  <si>
+    <t>PRP-4D57</t>
   </si>
   <si>
     <t>0B29</t>
   </si>
   <si>
-    <t xml:space="preserve">PIGTAIL OPTICO SIMPLEX SM SC UPC 3М</t>
+    <t>PIGTAIL OPTICO SIMPLEX SM SC UPC 3М</t>
+  </si>
+  <si>
+    <t>PRP-0B29</t>
   </si>
   <si>
     <t>3B01</t>
   </si>
   <si>
-    <t xml:space="preserve">PLAQUETA DE IDENTIFICAÇÃO</t>
+    <t>PLAQUETA DE IDENTIFICAÇÃO</t>
+  </si>
+  <si>
+    <t>PRP-3B01</t>
   </si>
   <si>
     <t>47B0</t>
   </si>
   <si>
-    <t xml:space="preserve">PONTO TERMINACAO OPTICO ROSETA</t>
+    <t>PONTO TERMINACAO OPTICO ROSETA</t>
+  </si>
+  <si>
+    <t>PRP-47B0</t>
   </si>
   <si>
     <t>A319</t>
   </si>
   <si>
-    <t xml:space="preserve">PORCA GAIOLA ENCAIXE 10-32</t>
+    <t>PORCA GAIOLA ENCAIXE 10-32</t>
+  </si>
+  <si>
+    <t>PRP-A319</t>
   </si>
   <si>
     <t>84B6</t>
   </si>
   <si>
-    <t xml:space="preserve">POWER CABLE AC I27V/22OV BLACK</t>
+    <t>POWER CABLE AC I27V/22OV BLACK</t>
+  </si>
+  <si>
+    <t>PRP-84B6</t>
   </si>
   <si>
     <t>6B75</t>
   </si>
   <si>
-    <t xml:space="preserve">PROTETOR DE EMENDA TERMOCONTRATIL PARA FIBRA OPTICA - DTC 105</t>
+    <t>PROTETOR DE EMENDA TERMOCONTRATIL PARA FIBRA OPTICA - DTC 105</t>
+  </si>
+  <si>
+    <t>PRP-6B75</t>
   </si>
   <si>
     <t>CBD9</t>
   </si>
   <si>
-    <t xml:space="preserve">PTO ROSETA 2P</t>
+    <t>PTO ROSETA 2P</t>
+  </si>
+  <si>
+    <t>PRP-CBD9</t>
   </si>
   <si>
     <t>4158</t>
   </si>
   <si>
-    <t xml:space="preserve">RACK PISO 19 44U X 970MM</t>
+    <t>RACK PISO 19 44U X 970MM</t>
+  </si>
+  <si>
+    <t>PRP-4158</t>
   </si>
   <si>
     <t>F82D</t>
   </si>
   <si>
-    <t xml:space="preserve">RESERVA GALVANIZADA DE CABO OPTICO POSTE</t>
+    <t>RESERVA GALVANIZADA DE CABO OPTICO POSTE</t>
+  </si>
+  <si>
+    <t>PRP-F82D</t>
   </si>
   <si>
     <t>F509</t>
   </si>
   <si>
-    <t xml:space="preserve">ROTEADOR ACCESS POINT AC PRO UBIQUITI 5GHZ</t>
+    <t>ROTEADOR ACCESS POINT AC PRO UBIQUITI 5GHZ</t>
+  </si>
+  <si>
+    <t>PRP-F509</t>
   </si>
   <si>
     <t>BE2F</t>
   </si>
   <si>
-    <t xml:space="preserve">ROTEADOR BORDA 3011 UIAS RM MIKROTIK 10P 1G</t>
+    <t>ROTEADOR BORDA 3011 UIAS RM MIKROTIK 10P 1G</t>
+  </si>
+  <si>
+    <t>PRP-BE2F</t>
   </si>
   <si>
     <t>7AB1</t>
   </si>
   <si>
-    <t xml:space="preserve">ROTEADOR BORDA 750GR3 MIKROTIK 5P 256MB</t>
+    <t>ROTEADOR BORDA 750GR3 MIKROTIK 5P 256MB</t>
+  </si>
+  <si>
+    <t>PRP-7AB1</t>
   </si>
   <si>
     <t>4A28</t>
   </si>
   <si>
-    <t xml:space="preserve">ROTEADOR BORDA 760IGS MIKROTIK HEX S</t>
+    <t>ROTEADOR BORDA 760IGS MIKROTIK HEX S</t>
+  </si>
+  <si>
+    <t>PRP-4A28</t>
   </si>
   <si>
     <t>C2AF</t>
   </si>
   <si>
-    <t xml:space="preserve">ROTEADOR BORDA CCR1016 MIKROTIK 12G</t>
+    <t>ROTEADOR BORDA CCR1016 MIKROTIK 12G</t>
+  </si>
+  <si>
+    <t>PRP-C2AF</t>
   </si>
   <si>
     <t>18D6</t>
   </si>
   <si>
-    <t xml:space="preserve">ROTEADOR BORDA CCR2004 MIKROTIK 16P 16G</t>
+    <t>ROTEADOR BORDA CCR2004 MIKROTIK 16P 16G</t>
+  </si>
+  <si>
+    <t>PRP-18D6</t>
   </si>
   <si>
     <t>D73C</t>
   </si>
   <si>
-    <t xml:space="preserve">ROTEADOR BORDA CCR1036 MIKROTIK 8G-2S+</t>
+    <t>ROTEADOR BORDA CCR1036 MIKROTIK 8G-2S+</t>
+  </si>
+  <si>
+    <t>PRP-D73C</t>
   </si>
   <si>
     <t>7CF6</t>
   </si>
   <si>
-    <t xml:space="preserve">ROTEADOR DE BORDA CCR2116_12G_4S MIKROTIK</t>
+    <t>ROTEADOR DE BORDA CCR2116_12G_4S MIKROTIK</t>
+  </si>
+  <si>
+    <t>PRP-7CF6</t>
   </si>
   <si>
     <t>8E1A</t>
   </si>
   <si>
-    <t xml:space="preserve">SFP + BIDI LR 10G 1270NM TX/1330NM RX 20KM LC</t>
+    <t>SFP + BIDI LR 10G 1270NM TX/1330NM RX 20KM LC</t>
+  </si>
+  <si>
+    <t>PRP-8E1A</t>
   </si>
   <si>
     <t>9A68</t>
   </si>
   <si>
-    <t xml:space="preserve">SFP BIDI 1.25G 1310NMTX/1550NMRX LC 20KM</t>
+    <t>SFP BIDI 1.25G 1310NMTX/1550NMRX LC 20KM</t>
+  </si>
+  <si>
+    <t>PRP-9A68</t>
   </si>
   <si>
     <t>8791</t>
   </si>
   <si>
-    <t xml:space="preserve">SFP BIDI 1.25G 1310NMTX/1550NMRX LC 40KM</t>
+    <t>SFP BIDI 1.25G 1310NMTX/1550NMRX LC 40KM</t>
+  </si>
+  <si>
+    <t>PRP-8791</t>
   </si>
   <si>
     <t>1DAC</t>
   </si>
   <si>
-    <t xml:space="preserve">SFP BIDI 1.25G 1310NMTX/1550NMRX SC 20KM</t>
+    <t>SFP BIDI 1.25G 1310NMTX/1550NMRX SC 20KM</t>
+  </si>
+  <si>
+    <t>PRP-1DAC</t>
   </si>
   <si>
     <t>5981</t>
   </si>
   <si>
-    <t xml:space="preserve">SFP BIDI 1.25G 1550NMTX/1310NMRX LC 20KM</t>
+    <t>SFP BIDI 1.25G 1550NMTX/1310NMRX LC 20KM</t>
+  </si>
+  <si>
+    <t>PRP-5981</t>
   </si>
   <si>
     <t>19DE</t>
   </si>
   <si>
-    <t xml:space="preserve">SFP BIDI 1.25G 1550NMTX/1310NMRX LC 40KM</t>
+    <t>SFP BIDI 1.25G 1550NMTX/1310NMRX LC 40KM</t>
+  </si>
+  <si>
+    <t>PRP-19DE</t>
   </si>
   <si>
     <t>F264</t>
   </si>
   <si>
-    <t xml:space="preserve">SFP BX BIDI 1550/1310 10KM LC</t>
+    <t>SFP BX BIDI 1550/1310 10KM LC</t>
+  </si>
+  <si>
+    <t>PRP-F264</t>
   </si>
   <si>
     <t>2CB5</t>
   </si>
   <si>
-    <t xml:space="preserve">SFP PRE-SFP-B35-20 1.25GB 1310TX/1550RX 20KM DDM</t>
+    <t>SFP PRE-SFP-B35-20 1.25GB 1310TX/1550RX 20KM DDM</t>
+  </si>
+  <si>
+    <t>PRP-2CB5</t>
   </si>
   <si>
     <t>EF35</t>
   </si>
   <si>
-    <t xml:space="preserve">SFP+ 10GBASE-LR</t>
+    <t>SFP+ 10GBASE-LR</t>
+  </si>
+  <si>
+    <t>PRP-EF35</t>
   </si>
   <si>
     <t>FAC3</t>
   </si>
   <si>
-    <t xml:space="preserve">SISTEMA RETENCAO CABO CIRCULAR DTC271</t>
+    <t>SISTEMA RETENCAO CABO CIRCULAR DTC271</t>
+  </si>
+  <si>
+    <t>PRP-FAC3</t>
   </si>
   <si>
     <t>EC1F</t>
   </si>
   <si>
-    <t xml:space="preserve">SPLITTER BALANCEADO 1:8 SC UPC DTC116</t>
+    <t>SPLITTER BALANCEADO 1:8 SC UPC DTC116</t>
+  </si>
+  <si>
+    <t>PRP-EC1F</t>
   </si>
   <si>
     <t>4A85</t>
   </si>
   <si>
-    <t xml:space="preserve">SPLITTER BALANCEADO 1X16 SC UPC</t>
+    <t>SPLITTER BALANCEADO 1X16 SC UPC</t>
+  </si>
+  <si>
+    <t>PRP-4A85</t>
   </si>
   <si>
     <t>4AE8</t>
   </si>
   <si>
-    <t xml:space="preserve">SPLITTER BALANCEADO I:4 SC UPC DTC116</t>
+    <t>SPLITTER BALANCEADO I:4 SC UPC DTC116</t>
+  </si>
+  <si>
+    <t>PRP-4AE8</t>
   </si>
   <si>
     <t>CF43</t>
   </si>
   <si>
-    <t xml:space="preserve">SUPORTE ANCORAGEM OLHAL RETO DTC227</t>
+    <t>SUPORTE ANCORAGEM OLHAL RETO DTC227</t>
+  </si>
+  <si>
+    <t>PRP-CF43</t>
   </si>
   <si>
     <t>2DE4</t>
   </si>
   <si>
-    <t xml:space="preserve">SUPORTE ANCORAGEM PASSAGEM ROLDANA DTC057</t>
+    <t>SUPORTE ANCORAGEM PASSAGEM ROLDANA DTC057</t>
+  </si>
+  <si>
+    <t>PRP-2DE4</t>
   </si>
   <si>
     <t>1BFA</t>
   </si>
   <si>
-    <t xml:space="preserve">SUPORTE DIELETRICO COMPACTO DE PASSAGEM PARA CABO OPTICO (SDR) - DTC 059</t>
+    <t>SUPORTE DIELETRICO COMPACTO DE PASSAGEM PARA CABO OPTICO (SDR) - DTC 059</t>
+  </si>
+  <si>
+    <t>PRP-1BFA</t>
   </si>
   <si>
     <t>CBF7</t>
   </si>
   <si>
-    <t xml:space="preserve">SUPORTE DIELETRICO COMPАСТО PASSAGEM DTC059</t>
+    <t>SUPORTE DIELETRICO COMPАСТО PASSAGEM DTC059</t>
+  </si>
+  <si>
+    <t>PRP-CBF7</t>
   </si>
   <si>
     <t>42E1</t>
   </si>
   <si>
-    <t xml:space="preserve">SUPORTE RESERVA CABO CORDOALHA DTC136</t>
+    <t>SUPORTE RESERVA CABO CORDOALHA DTC136</t>
+  </si>
+  <si>
+    <t>PRP-42E1</t>
   </si>
   <si>
     <t>B59F</t>
   </si>
   <si>
-    <t xml:space="preserve">SUPORTE ROLDANA ANCORAGEM CABO ASU DTC058</t>
+    <t>SUPORTE ROLDANA ANCORAGEM CABO ASU DTC058</t>
+  </si>
+  <si>
+    <t>PRP-B59F</t>
   </si>
   <si>
     <t>D1C8</t>
   </si>
   <si>
-    <t xml:space="preserve">SUPORTE SDA CABO FIBRA OPTICA</t>
+    <t>SUPORTE SDA CABO FIBRA OPTICA</t>
+  </si>
+  <si>
+    <t>PRP-D1C8</t>
   </si>
   <si>
     <t>5C7F</t>
   </si>
   <si>
-    <t xml:space="preserve">SUPORTE UNIVERSAL PASSAGEM ANCORAGEM CABO SUPA</t>
+    <t>SUPORTE UNIVERSAL PASSAGEM ANCORAGEM CABO SUPA</t>
+  </si>
+  <si>
+    <t>PRP-5C7F</t>
   </si>
   <si>
     <t>4DBA</t>
   </si>
   <si>
-    <t xml:space="preserve">SWITCH DM2104-G2 EDD 1G</t>
+    <t>SWITCH DM2104-G2 EDD 1G</t>
+  </si>
+  <si>
+    <t>PRP-4DBA</t>
   </si>
   <si>
     <t>2180</t>
   </si>
   <si>
-    <t xml:space="preserve">SWITCH DM2301 4GT 4GX</t>
+    <t>SWITCH DM2301 4GT 4GX</t>
+  </si>
+  <si>
+    <t>PRP-2180</t>
   </si>
   <si>
     <t>C986</t>
   </si>
   <si>
-    <t xml:space="preserve">SWITCH DM4370 4GT 4XS</t>
+    <t>SWITCH DM4370 4GT 4XS</t>
+  </si>
+  <si>
+    <t>PRP-C986</t>
   </si>
   <si>
     <t>6D10</t>
   </si>
   <si>
-    <t xml:space="preserve">SWITCH HUAWEI S6730 H24X6C</t>
+    <t>SWITCH HUAWEI S6730 H24X6C</t>
+  </si>
+  <si>
+    <t>PRP-6D10</t>
   </si>
   <si>
     <t>052A</t>
   </si>
   <si>
-    <t xml:space="preserve">TERMINADOR OPTICO EXTERNO 6FO TOE DTC302</t>
+    <t>TERMINADOR OPTICO EXTERNO 6FO TOE DTC302</t>
+  </si>
+  <si>
+    <t>PRP-052A</t>
   </si>
   <si>
     <t>B6C3</t>
   </si>
   <si>
-    <t xml:space="preserve">TERMINAL ISOLADO PINO CHATO 35MM</t>
+    <t>TERMINAL ISOLADO PINO CHATO 35MM</t>
+  </si>
+  <si>
+    <t>PRP-B6C3</t>
   </si>
   <si>
     <t>486C</t>
   </si>
   <si>
-    <t xml:space="preserve">TUBO GALVANIZADO NBR5580 2 1/2</t>
+    <t>TUBO GALVANIZADO NBR5580 2 1/2</t>
+  </si>
+  <si>
+    <t>PRP-486C</t>
   </si>
 </sst>
 </file>
@@ -1663,1467 +2209,2014 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultColWidth="11.220000000000001" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="7.375"/>
-    <col customWidth="1" min="2" max="2" width="62.219999999999999"/>
+    <col customWidth="1" min="1" max="1" width="12"/>
+    <col customWidth="1" min="2" max="2" width="62"/>
+    <col customWidth="1" min="3" max="3" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5">
-      <c r="A1" s="1" t="s">
+    <row r="1">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" ht="16.5">
-      <c r="A2" s="3" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" ht="16.5">
-      <c r="A3" s="3" t="s">
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" ht="16.5">
-      <c r="A4" s="3" t="s">
+    <row r="3">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" ht="16.5">
-      <c r="A5" s="3" t="s">
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="3" t="s">
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" ht="16.5">
-      <c r="A6" s="3" t="s">
+      <c r="B4" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" ht="16.5">
-      <c r="A7" s="3" t="s">
+    <row r="5">
+      <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B5" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" ht="16.5">
-      <c r="A8" s="3" t="s">
+      <c r="C5" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="3" t="s">
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" ht="16.5">
-      <c r="A9" s="3" t="s">
+      <c r="B6" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" ht="16.5">
-      <c r="A10" s="3" t="s">
+    <row r="7">
+      <c r="A7" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B7" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" ht="16.5">
-      <c r="A11" s="3" t="s">
+      <c r="C7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="3" t="s">
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="12" ht="16.5">
-      <c r="A12" s="3" t="s">
+      <c r="B8" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="C8" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="13" ht="16.5">
-      <c r="A13" s="3" t="s">
+    <row r="9">
+      <c r="A9" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B9" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="14" ht="16.5">
-      <c r="A14" s="3" t="s">
+      <c r="C9" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="3" t="s">
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="15" ht="16.5">
-      <c r="A15" s="3" t="s">
+      <c r="B10" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="C10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" ht="16.5">
-      <c r="A16" s="3" t="s">
+    <row r="11">
+      <c r="A11" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B11" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="17" ht="16.5">
-      <c r="A17" s="3" t="s">
+      <c r="C11" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="3" t="s">
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="18" ht="16.5">
-      <c r="A18" s="3" t="s">
+      <c r="B12" t="s">
         <v>34</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="C12" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="19" ht="16.5">
-      <c r="A19" s="3" t="s">
+    <row r="13">
+      <c r="A13" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B13" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="20" ht="16.5">
-      <c r="A20" s="3" t="s">
+      <c r="C13" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="3" t="s">
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="3" t="s">
+      <c r="B14" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="C14" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="3" t="s">
+    <row r="15">
+      <c r="A15" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B15" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="3" t="s">
+      <c r="C15" t="s">
         <v>44</v>
       </c>
-      <c r="B23" s="3" t="s">
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="3" t="s">
+      <c r="B16" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="C16" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="3" t="s">
+    <row r="17">
+      <c r="A17" t="s">
         <v>48</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B17" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="3" t="s">
+      <c r="C17" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="3" t="s">
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="3" t="s">
+      <c r="B18" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="C18" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="3" t="s">
+    <row r="19">
+      <c r="A19" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B19" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="3" t="s">
+      <c r="C19" t="s">
         <v>56</v>
       </c>
-      <c r="B29" s="4" t="s">
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="3" t="s">
+      <c r="B20" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="C20" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="3" t="s">
+    <row r="21">
+      <c r="A21" t="s">
         <v>60</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B21" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="3" t="s">
+      <c r="C21" t="s">
         <v>62</v>
       </c>
-      <c r="B32" s="3" t="s">
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="3" t="s">
+      <c r="B22" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="C22" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="3" t="s">
+    <row r="23">
+      <c r="A23" t="s">
         <v>66</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B23" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="3" t="s">
+      <c r="C23" t="s">
         <v>68</v>
       </c>
-      <c r="B35" s="3" t="s">
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="3" t="s">
+      <c r="B24" t="s">
         <v>70</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="C24" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="3" t="s">
+    <row r="25">
+      <c r="A25" t="s">
         <v>72</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B25" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="3" t="s">
+      <c r="C25" t="s">
         <v>74</v>
       </c>
-      <c r="B38" s="3" t="s">
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="3" t="s">
+      <c r="B26" t="s">
         <v>76</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="C26" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="3" t="s">
+    <row r="27">
+      <c r="A27" t="s">
         <v>78</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="B27" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="3" t="s">
+      <c r="C27" t="s">
         <v>80</v>
       </c>
-      <c r="B41" s="3" t="s">
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="3" t="s">
+      <c r="B28" t="s">
         <v>82</v>
       </c>
-      <c r="B42" s="3" t="s">
+      <c r="C28" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="3" t="s">
+    <row r="29">
+      <c r="A29" t="s">
         <v>84</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="B29" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="3" t="s">
+      <c r="C29" t="s">
         <v>86</v>
       </c>
-      <c r="B44" s="3" t="s">
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="3" t="s">
+      <c r="B30" t="s">
         <v>88</v>
       </c>
-      <c r="B45" s="3" t="s">
+      <c r="C30" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="3" t="s">
+    <row r="31">
+      <c r="A31" t="s">
         <v>90</v>
       </c>
-      <c r="B46" s="3" t="s">
+      <c r="B31" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="3" t="s">
+      <c r="C31" t="s">
         <v>92</v>
       </c>
-      <c r="B47" s="3" t="s">
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="3" t="s">
+      <c r="B32" t="s">
         <v>94</v>
       </c>
-      <c r="B48" s="3" t="s">
+      <c r="C32" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="3" t="s">
+    <row r="33">
+      <c r="A33" t="s">
         <v>96</v>
       </c>
-      <c r="B49" s="3" t="s">
+      <c r="B33" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="3" t="s">
+      <c r="C33" t="s">
         <v>98</v>
       </c>
-      <c r="B50" s="3" t="s">
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="51" ht="15.75" customHeight="1">
-      <c r="A51" s="3" t="s">
+      <c r="B34" t="s">
         <v>100</v>
       </c>
-      <c r="B51" s="3" t="s">
+      <c r="C34" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="3" t="s">
+    <row r="35">
+      <c r="A35" t="s">
         <v>102</v>
       </c>
-      <c r="B52" s="3" t="s">
+      <c r="B35" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="3" t="s">
+      <c r="C35" t="s">
         <v>104</v>
       </c>
-      <c r="B53" s="3" t="s">
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="54" ht="15.75" customHeight="1">
-      <c r="A54" s="3" t="s">
+      <c r="B36" t="s">
         <v>106</v>
       </c>
-      <c r="B54" s="3" t="s">
+      <c r="C36" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="55" ht="15.75" customHeight="1">
-      <c r="A55" s="3" t="s">
+    <row r="37">
+      <c r="A37" t="s">
         <v>108</v>
       </c>
-      <c r="B55" s="3" t="s">
+      <c r="B37" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="3" t="s">
+      <c r="C37" t="s">
         <v>110</v>
       </c>
-      <c r="B56" s="3" t="s">
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="3" t="s">
+      <c r="B38" t="s">
         <v>112</v>
       </c>
-      <c r="B57" s="3" t="s">
+      <c r="C38" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="3" t="s">
+    <row r="39">
+      <c r="A39" t="s">
         <v>114</v>
       </c>
-      <c r="B58" s="3" t="s">
+      <c r="B39" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="59" ht="15.75" customHeight="1">
-      <c r="A59" s="3" t="s">
+      <c r="C39" t="s">
         <v>116</v>
       </c>
-      <c r="B59" s="3" t="s">
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="60" ht="15.75" customHeight="1">
-      <c r="A60" s="3" t="s">
+      <c r="B40" t="s">
         <v>118</v>
       </c>
-      <c r="B60" s="3" t="s">
+      <c r="C40" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="61" ht="15.75" customHeight="1">
-      <c r="A61" s="3" t="s">
+    <row r="41">
+      <c r="A41" t="s">
         <v>120</v>
       </c>
-      <c r="B61" s="3" t="s">
+      <c r="B41" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="62" ht="15.75" customHeight="1">
-      <c r="A62" s="3" t="s">
+      <c r="C41" t="s">
         <v>122</v>
       </c>
-      <c r="B62" s="3" t="s">
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="63" ht="15.75" customHeight="1">
-      <c r="A63" s="3" t="s">
+      <c r="B42" t="s">
         <v>124</v>
       </c>
-      <c r="B63" s="3" t="s">
+      <c r="C42" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="64" ht="15.75" customHeight="1">
-      <c r="A64" s="3" t="s">
+    <row r="43">
+      <c r="A43" t="s">
         <v>126</v>
       </c>
-      <c r="B64" s="3" t="s">
+      <c r="B43" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="65" ht="15.75" customHeight="1">
-      <c r="A65" s="3" t="s">
+      <c r="C43" t="s">
         <v>128</v>
       </c>
-      <c r="B65" s="3" t="s">
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="66" ht="15.75" customHeight="1">
-      <c r="A66" s="3" t="s">
+      <c r="B44" t="s">
         <v>130</v>
       </c>
-      <c r="B66" s="3" t="s">
+      <c r="C44" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="67" ht="15.75" customHeight="1">
-      <c r="A67" s="3" t="s">
+    <row r="45">
+      <c r="A45" t="s">
         <v>132</v>
       </c>
-      <c r="B67" s="3" t="s">
+      <c r="B45" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="68" ht="15.75" customHeight="1">
-      <c r="A68" s="3" t="s">
+      <c r="C45" t="s">
         <v>134</v>
       </c>
-      <c r="B68" s="3" t="s">
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="69" ht="15.75" customHeight="1">
-      <c r="A69" s="3" t="s">
+      <c r="B46" t="s">
         <v>136</v>
       </c>
-      <c r="B69" s="3" t="s">
+      <c r="C46" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="70" ht="15.75" customHeight="1">
-      <c r="A70" s="3" t="s">
+    <row r="47">
+      <c r="A47" t="s">
         <v>138</v>
       </c>
-      <c r="B70" s="3" t="s">
+      <c r="B47" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="71" ht="15.75" customHeight="1">
-      <c r="A71" s="3" t="s">
+      <c r="C47" t="s">
         <v>140</v>
       </c>
-      <c r="B71" s="3" t="s">
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="72" ht="15.75" customHeight="1">
-      <c r="A72" s="3" t="s">
+      <c r="B48" t="s">
         <v>142</v>
       </c>
-      <c r="B72" s="3" t="s">
+      <c r="C48" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="73" ht="15.75" customHeight="1">
-      <c r="A73" s="3" t="s">
+    <row r="49">
+      <c r="A49" t="s">
         <v>144</v>
       </c>
-      <c r="B73" s="3" t="s">
+      <c r="B49" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="74" ht="15.75" customHeight="1">
-      <c r="A74" s="3" t="s">
+      <c r="C49" t="s">
         <v>146</v>
       </c>
-      <c r="B74" s="3" t="s">
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="75" ht="15.75" customHeight="1">
-      <c r="A75" s="3" t="s">
+      <c r="B50" t="s">
         <v>148</v>
       </c>
-      <c r="B75" s="3" t="s">
+      <c r="C50" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="76" ht="15.75" customHeight="1">
-      <c r="A76" s="3" t="s">
+    <row r="51">
+      <c r="A51" t="s">
         <v>150</v>
       </c>
-      <c r="B76" s="3" t="s">
+      <c r="B51" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="77" ht="15.75" customHeight="1">
-      <c r="A77" s="3" t="s">
+      <c r="C51" t="s">
         <v>152</v>
       </c>
-      <c r="B77" s="3" t="s">
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="78" ht="15.75" customHeight="1">
-      <c r="A78" s="3" t="s">
+      <c r="B52" t="s">
         <v>154</v>
       </c>
-      <c r="B78" s="3" t="s">
+      <c r="C52" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="79" ht="15.75" customHeight="1">
-      <c r="A79" s="3" t="s">
+    <row r="53">
+      <c r="A53" t="s">
         <v>156</v>
       </c>
-      <c r="B79" s="3" t="s">
+      <c r="B53" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="80" ht="15.75" customHeight="1">
-      <c r="A80" s="3" t="s">
+      <c r="C53" t="s">
         <v>158</v>
       </c>
-      <c r="B80" s="3" t="s">
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="81" ht="15.75" customHeight="1">
-      <c r="A81" s="3" t="s">
+      <c r="B54" t="s">
         <v>160</v>
       </c>
-      <c r="B81" s="3" t="s">
+      <c r="C54" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="82" ht="15.75" customHeight="1">
-      <c r="A82" s="3" t="s">
+    <row r="55">
+      <c r="A55" t="s">
         <v>162</v>
       </c>
-      <c r="B82" s="3" t="s">
+      <c r="B55" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="83" ht="15.75" customHeight="1">
-      <c r="A83" s="3" t="s">
+      <c r="C55" t="s">
         <v>164</v>
       </c>
-      <c r="B83" s="3" t="s">
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="84" ht="15.75" customHeight="1">
-      <c r="A84" s="3" t="s">
+      <c r="B56" t="s">
         <v>166</v>
       </c>
-      <c r="B84" s="3" t="s">
+      <c r="C56" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="85" ht="15.75" customHeight="1">
-      <c r="A85" s="3" t="s">
+    <row r="57">
+      <c r="A57" t="s">
         <v>168</v>
       </c>
-      <c r="B85" s="3" t="s">
+      <c r="B57" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="86" ht="15.75" customHeight="1">
-      <c r="A86" s="3" t="s">
+      <c r="C57" t="s">
         <v>170</v>
       </c>
-      <c r="B86" s="3" t="s">
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="87" ht="15.75" customHeight="1">
-      <c r="A87" s="3" t="s">
+      <c r="B58" t="s">
         <v>172</v>
       </c>
-      <c r="B87" s="3" t="s">
+      <c r="C58" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="88" ht="15.75" customHeight="1">
-      <c r="A88" s="3" t="s">
+    <row r="59">
+      <c r="A59" t="s">
         <v>174</v>
       </c>
-      <c r="B88" s="3" t="s">
+      <c r="B59" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="89" ht="15.75" customHeight="1">
-      <c r="A89" s="3" t="s">
+      <c r="C59" t="s">
         <v>176</v>
       </c>
-      <c r="B89" s="3" t="s">
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="90" ht="15.75" customHeight="1">
-      <c r="A90" s="3" t="s">
+      <c r="B60" t="s">
         <v>178</v>
       </c>
-      <c r="B90" s="3" t="s">
+      <c r="C60" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="91" ht="15.75" customHeight="1">
-      <c r="A91" s="3" t="s">
+    <row r="61">
+      <c r="A61" t="s">
         <v>180</v>
       </c>
-      <c r="B91" s="3" t="s">
+      <c r="B61" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="92" ht="15.75" customHeight="1">
-      <c r="A92" s="3" t="s">
+      <c r="C61" t="s">
         <v>182</v>
       </c>
-      <c r="B92" s="3" t="s">
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="93" ht="15.75" customHeight="1">
-      <c r="A93" s="3" t="s">
+      <c r="B62" t="s">
         <v>184</v>
       </c>
-      <c r="B93" s="3" t="s">
+      <c r="C62" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="94" ht="15.75" customHeight="1">
-      <c r="A94" s="3" t="s">
+    <row r="63">
+      <c r="A63" t="s">
         <v>186</v>
       </c>
-      <c r="B94" s="3" t="s">
+      <c r="B63" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="95" ht="15.75" customHeight="1">
-      <c r="A95" s="3" t="s">
+      <c r="C63" t="s">
         <v>188</v>
       </c>
-      <c r="B95" s="3" t="s">
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="96" ht="15.75" customHeight="1">
-      <c r="A96" s="3" t="s">
+      <c r="B64" t="s">
         <v>190</v>
       </c>
-      <c r="B96" s="3" t="s">
+      <c r="C64" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="97" ht="15.75" customHeight="1">
-      <c r="A97" s="3" t="s">
+    <row r="65">
+      <c r="A65" t="s">
         <v>192</v>
       </c>
-      <c r="B97" s="3" t="s">
+      <c r="B65" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="98" ht="15.75" customHeight="1">
-      <c r="A98" s="3" t="s">
+      <c r="C65" t="s">
         <v>194</v>
       </c>
-      <c r="B98" s="3" t="s">
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="99" ht="15.75" customHeight="1">
-      <c r="A99" s="3" t="s">
+      <c r="B66" t="s">
         <v>196</v>
       </c>
-      <c r="B99" s="3" t="s">
+      <c r="C66" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="100" ht="15.75" customHeight="1">
-      <c r="A100" s="3" t="s">
+    <row r="67">
+      <c r="A67" t="s">
         <v>198</v>
       </c>
-      <c r="B100" s="3" t="s">
+      <c r="B67" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="101" ht="15.75" customHeight="1">
-      <c r="A101" s="3" t="s">
+      <c r="C67" t="s">
         <v>200</v>
       </c>
-      <c r="B101" s="4" t="s">
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="102" ht="15.75" customHeight="1">
-      <c r="A102" s="3" t="s">
+      <c r="B68" t="s">
         <v>202</v>
       </c>
-      <c r="B102" s="3" t="s">
+      <c r="C68" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="103" ht="15.75" customHeight="1">
-      <c r="A103" s="3" t="s">
+    <row r="69">
+      <c r="A69" t="s">
         <v>204</v>
       </c>
-      <c r="B103" s="3" t="s">
+      <c r="B69" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="104" ht="15.75" customHeight="1">
-      <c r="A104" s="3" t="s">
+      <c r="C69" t="s">
         <v>206</v>
       </c>
-      <c r="B104" s="3" t="s">
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="105" ht="15.75" customHeight="1">
-      <c r="A105" s="3" t="s">
+      <c r="B70" t="s">
         <v>208</v>
       </c>
-      <c r="B105" s="3" t="s">
+      <c r="C70" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="106" ht="15.75" customHeight="1">
-      <c r="A106" s="3" t="s">
+    <row r="71">
+      <c r="A71" t="s">
         <v>210</v>
       </c>
-      <c r="B106" s="3" t="s">
+      <c r="B71" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="107" ht="15.75" customHeight="1">
-      <c r="A107" s="3" t="s">
+      <c r="C71" t="s">
         <v>212</v>
       </c>
-      <c r="B107" s="3" t="s">
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="108" ht="15.75" customHeight="1">
-      <c r="A108" s="3" t="s">
+      <c r="B72" t="s">
         <v>214</v>
       </c>
-      <c r="B108" s="3" t="s">
+      <c r="C72" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="109" ht="15.75" customHeight="1">
-      <c r="A109" s="3" t="s">
+    <row r="73">
+      <c r="A73" t="s">
         <v>216</v>
       </c>
-      <c r="B109" s="3" t="s">
+      <c r="B73" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="110" ht="15.75" customHeight="1">
-      <c r="A110" s="3" t="s">
+      <c r="C73" t="s">
         <v>218</v>
       </c>
-      <c r="B110" s="3" t="s">
+    </row>
+    <row r="74">
+      <c r="A74" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="111" ht="15.75" customHeight="1">
-      <c r="A111" s="3" t="s">
+      <c r="B74" t="s">
         <v>220</v>
       </c>
-      <c r="B111" s="3" t="s">
+      <c r="C74" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="112" ht="15.75" customHeight="1">
-      <c r="A112" s="3" t="s">
+    <row r="75">
+      <c r="A75" t="s">
         <v>222</v>
       </c>
-      <c r="B112" s="3" t="s">
+      <c r="B75" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="113" ht="15.75" customHeight="1">
-      <c r="A113" s="3" t="s">
+      <c r="C75" t="s">
         <v>224</v>
       </c>
-      <c r="B113" s="3" t="s">
+    </row>
+    <row r="76">
+      <c r="A76" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="114" ht="15.75" customHeight="1">
-      <c r="A114" s="3" t="s">
+      <c r="B76" t="s">
         <v>226</v>
       </c>
-      <c r="B114" s="3" t="s">
+      <c r="C76" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="115" ht="15.75" customHeight="1">
-      <c r="A115" s="3" t="s">
+    <row r="77">
+      <c r="A77" t="s">
         <v>228</v>
       </c>
-      <c r="B115" s="3" t="s">
+      <c r="B77" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="116" ht="15.75" customHeight="1">
-      <c r="A116" s="3" t="s">
+      <c r="C77" t="s">
         <v>230</v>
       </c>
-      <c r="B116" s="3" t="s">
+    </row>
+    <row r="78">
+      <c r="A78" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="117" ht="15.75" customHeight="1">
-      <c r="A117" s="3" t="s">
+      <c r="B78" t="s">
         <v>232</v>
       </c>
-      <c r="B117" s="3" t="s">
+      <c r="C78" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="118" ht="15.75" customHeight="1">
-      <c r="A118" s="3" t="s">
+    <row r="79">
+      <c r="A79" t="s">
         <v>234</v>
       </c>
-      <c r="B118" s="3" t="s">
+      <c r="B79" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="119" ht="15.75" customHeight="1">
-      <c r="A119" s="3" t="s">
+      <c r="C79" t="s">
         <v>236</v>
       </c>
-      <c r="B119" s="3" t="s">
+    </row>
+    <row r="80">
+      <c r="A80" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="120" ht="15.75" customHeight="1">
-      <c r="A120" s="3" t="s">
+      <c r="B80" t="s">
         <v>238</v>
       </c>
-      <c r="B120" s="3" t="s">
+      <c r="C80" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="121" ht="15.75" customHeight="1">
-      <c r="A121" s="3" t="s">
+    <row r="81">
+      <c r="A81" t="s">
         <v>240</v>
       </c>
-      <c r="B121" s="3" t="s">
+      <c r="B81" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="122" ht="15.75" customHeight="1">
-      <c r="A122" s="3" t="s">
+      <c r="C81" t="s">
         <v>242</v>
       </c>
-      <c r="B122" s="3" t="s">
+    </row>
+    <row r="82">
+      <c r="A82" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="123" ht="15.75" customHeight="1">
-      <c r="A123" s="3" t="s">
+      <c r="B82" t="s">
         <v>244</v>
       </c>
-      <c r="B123" s="3" t="s">
+      <c r="C82" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="124" ht="15.75" customHeight="1">
-      <c r="A124" s="3" t="s">
+    <row r="83">
+      <c r="A83" t="s">
         <v>246</v>
       </c>
-      <c r="B124" s="3" t="s">
+      <c r="B83" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="125" ht="15.75" customHeight="1">
-      <c r="A125" s="3" t="s">
+      <c r="C83" t="s">
         <v>248</v>
       </c>
-      <c r="B125" s="3" t="s">
+    </row>
+    <row r="84">
+      <c r="A84" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="126" ht="15.75" customHeight="1">
-      <c r="A126" s="3" t="s">
+      <c r="B84" t="s">
         <v>250</v>
       </c>
-      <c r="B126" s="3" t="s">
+      <c r="C84" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="127" ht="15.75" customHeight="1">
-      <c r="A127" s="3" t="s">
+    <row r="85">
+      <c r="A85" t="s">
         <v>252</v>
       </c>
-      <c r="B127" s="3" t="s">
+      <c r="B85" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="128" ht="15.75" customHeight="1">
-      <c r="A128" s="3" t="s">
+      <c r="C85" t="s">
         <v>254</v>
       </c>
-      <c r="B128" s="3" t="s">
+    </row>
+    <row r="86">
+      <c r="A86" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="129" ht="15.75" customHeight="1">
-      <c r="A129" s="3" t="s">
+      <c r="B86" t="s">
         <v>256</v>
       </c>
-      <c r="B129" s="3" t="s">
+      <c r="C86" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="130" ht="15.75" customHeight="1">
-      <c r="A130" s="3" t="s">
+    <row r="87">
+      <c r="A87" t="s">
         <v>258</v>
       </c>
-      <c r="B130" s="3" t="s">
+      <c r="B87" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="131" ht="15.75" customHeight="1">
-      <c r="A131" s="3" t="s">
+      <c r="C87" t="s">
         <v>260</v>
       </c>
-      <c r="B131" s="3" t="s">
+    </row>
+    <row r="88">
+      <c r="A88" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="132" ht="15.75" customHeight="1">
-      <c r="A132" s="3" t="s">
+      <c r="B88" t="s">
         <v>262</v>
       </c>
-      <c r="B132" s="3" t="s">
+      <c r="C88" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="133" ht="15.75" customHeight="1">
-      <c r="A133" s="3" t="s">
+    <row r="89">
+      <c r="A89" t="s">
         <v>264</v>
       </c>
-      <c r="B133" s="3" t="s">
+      <c r="B89" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="134" ht="15.75" customHeight="1">
-      <c r="A134" s="3" t="s">
+      <c r="C89" t="s">
         <v>266</v>
       </c>
-      <c r="B134" s="3" t="s">
+    </row>
+    <row r="90">
+      <c r="A90" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="135" ht="15.75" customHeight="1">
-      <c r="A135" s="3" t="s">
+      <c r="B90" t="s">
         <v>268</v>
       </c>
-      <c r="B135" s="3" t="s">
+      <c r="C90" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="136" ht="15.75" customHeight="1">
-      <c r="A136" s="3" t="s">
+    <row r="91">
+      <c r="A91" t="s">
         <v>270</v>
       </c>
-      <c r="B136" s="3" t="s">
+      <c r="B91" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="137" ht="15.75" customHeight="1">
-      <c r="A137" s="3" t="s">
+      <c r="C91" t="s">
         <v>272</v>
       </c>
-      <c r="B137" s="3" t="s">
+    </row>
+    <row r="92">
+      <c r="A92" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="138" ht="15.75" customHeight="1">
-      <c r="A138" s="3" t="s">
+      <c r="B92" t="s">
         <v>274</v>
       </c>
-      <c r="B138" s="3" t="s">
+      <c r="C92" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="139" ht="15.75" customHeight="1">
-      <c r="A139" s="3" t="s">
+    <row r="93">
+      <c r="A93" t="s">
         <v>276</v>
       </c>
-      <c r="B139" s="3" t="s">
+      <c r="B93" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="140" ht="15.75" customHeight="1">
-      <c r="A140" s="3" t="s">
+      <c r="C93" t="s">
         <v>278</v>
       </c>
-      <c r="B140" s="3" t="s">
+    </row>
+    <row r="94">
+      <c r="A94" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="141" ht="15.75" customHeight="1">
-      <c r="A141" s="3" t="s">
+      <c r="B94" t="s">
         <v>280</v>
       </c>
-      <c r="B141" s="3" t="s">
+      <c r="C94" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="142" ht="15.75" customHeight="1">
-      <c r="A142" s="3" t="s">
+    <row r="95">
+      <c r="A95" t="s">
         <v>282</v>
       </c>
-      <c r="B142" s="3" t="s">
+      <c r="B95" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="143" ht="15.75" customHeight="1">
-      <c r="A143" s="3" t="s">
+      <c r="C95" t="s">
         <v>284</v>
       </c>
-      <c r="B143" s="3" t="s">
+    </row>
+    <row r="96">
+      <c r="A96" t="s">
         <v>285</v>
       </c>
-    </row>
-    <row r="144" ht="15.75" customHeight="1">
-      <c r="A144" s="3" t="s">
+      <c r="B96" t="s">
         <v>286</v>
       </c>
-      <c r="B144" s="3" t="s">
+      <c r="C96" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="145" ht="15.75" customHeight="1">
-      <c r="A145" s="3" t="s">
+    <row r="97">
+      <c r="A97" t="s">
         <v>288</v>
       </c>
-      <c r="B145" s="3" t="s">
+      <c r="B97" t="s">
         <v>289</v>
       </c>
-    </row>
-    <row r="146" ht="15.75" customHeight="1">
-      <c r="A146" s="3" t="s">
+      <c r="C97" t="s">
         <v>290</v>
       </c>
-      <c r="B146" s="3" t="s">
+    </row>
+    <row r="98">
+      <c r="A98" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="147" ht="15.75" customHeight="1">
-      <c r="A147" s="3" t="s">
+      <c r="B98" t="s">
         <v>292</v>
       </c>
-      <c r="B147" s="3" t="s">
+      <c r="C98" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="148" ht="15.75" customHeight="1">
-      <c r="A148" s="3" t="s">
+    <row r="99">
+      <c r="A99" t="s">
         <v>294</v>
       </c>
-      <c r="B148" s="3" t="s">
+      <c r="B99" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="149" ht="15.75" customHeight="1">
-      <c r="A149" s="3" t="s">
+      <c r="C99" t="s">
         <v>296</v>
       </c>
-      <c r="B149" s="3" t="s">
+    </row>
+    <row r="100">
+      <c r="A100" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="150" ht="15.75" customHeight="1">
-      <c r="A150" s="3" t="s">
+      <c r="B100" t="s">
         <v>298</v>
       </c>
-      <c r="B150" s="3" t="s">
+      <c r="C100" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="151" ht="15.75" customHeight="1">
-      <c r="A151" s="3" t="s">
+    <row r="101">
+      <c r="A101" t="s">
         <v>300</v>
       </c>
-      <c r="B151" s="3" t="s">
+      <c r="B101" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="152" ht="15.75" customHeight="1">
-      <c r="A152" s="3" t="s">
+      <c r="C101" t="s">
         <v>302</v>
       </c>
-      <c r="B152" s="3" t="s">
+    </row>
+    <row r="102">
+      <c r="A102" t="s">
         <v>303</v>
       </c>
-    </row>
-    <row r="153" ht="15.75" customHeight="1">
-      <c r="A153" s="3" t="s">
+      <c r="B102" t="s">
         <v>304</v>
       </c>
-      <c r="B153" s="4" t="s">
+      <c r="C102" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="154" ht="15.75" customHeight="1">
-      <c r="A154" s="3" t="s">
+    <row r="103">
+      <c r="A103" t="s">
         <v>306</v>
       </c>
-      <c r="B154" s="3" t="s">
+      <c r="B103" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="155" ht="15.75" customHeight="1">
-      <c r="A155" s="3" t="s">
+      <c r="C103" t="s">
         <v>308</v>
       </c>
-      <c r="B155" s="3" t="s">
+    </row>
+    <row r="104">
+      <c r="A104" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="156" ht="15.75" customHeight="1">
-      <c r="A156" s="3" t="s">
+      <c r="B104" t="s">
         <v>310</v>
       </c>
-      <c r="B156" s="3" t="s">
+      <c r="C104" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="157" ht="15.75" customHeight="1">
-      <c r="A157" s="3" t="s">
+    <row r="105">
+      <c r="A105" t="s">
         <v>312</v>
       </c>
-      <c r="B157" s="3" t="s">
+      <c r="B105" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="158" ht="15.75" customHeight="1">
-      <c r="A158" s="3" t="s">
+      <c r="C105" t="s">
         <v>314</v>
       </c>
-      <c r="B158" s="3" t="s">
+    </row>
+    <row r="106">
+      <c r="A106" t="s">
         <v>315</v>
       </c>
-    </row>
-    <row r="159" ht="15.75" customHeight="1">
-      <c r="A159" s="3" t="s">
+      <c r="B106" t="s">
         <v>316</v>
       </c>
-      <c r="B159" s="3" t="s">
+      <c r="C106" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="160" ht="15.75" customHeight="1">
-      <c r="A160" s="3" t="s">
+    <row r="107">
+      <c r="A107" t="s">
         <v>318</v>
       </c>
-      <c r="B160" s="3" t="s">
+      <c r="B107" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="161" ht="15.75" customHeight="1">
-      <c r="A161" s="3" t="s">
+      <c r="C107" t="s">
         <v>320</v>
       </c>
-      <c r="B161" s="3" t="s">
+    </row>
+    <row r="108">
+      <c r="A108" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="162" ht="15.75" customHeight="1">
-      <c r="A162" s="3" t="s">
+      <c r="B108" t="s">
         <v>322</v>
       </c>
-      <c r="B162" s="3" t="s">
+      <c r="C108" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="163" ht="15.75" customHeight="1">
-      <c r="A163" s="3" t="s">
+    <row r="109">
+      <c r="A109" t="s">
         <v>324</v>
       </c>
-      <c r="B163" s="3" t="s">
+      <c r="B109" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="164" ht="15.75" customHeight="1">
-      <c r="A164" s="3" t="s">
+      <c r="C109" t="s">
         <v>326</v>
       </c>
-      <c r="B164" s="3" t="s">
+    </row>
+    <row r="110">
+      <c r="A110" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="165" ht="15.75" customHeight="1">
-      <c r="A165" s="3" t="s">
+      <c r="B110" t="s">
         <v>328</v>
       </c>
-      <c r="B165" s="4" t="s">
+      <c r="C110" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="166" ht="15.75" customHeight="1">
-      <c r="A166" s="3" t="s">
+    <row r="111">
+      <c r="A111" t="s">
         <v>330</v>
       </c>
-      <c r="B166" s="3" t="s">
+      <c r="B111" t="s">
         <v>331</v>
       </c>
-    </row>
-    <row r="167" ht="15.75" customHeight="1">
-      <c r="A167" s="3" t="s">
+      <c r="C111" t="s">
         <v>332</v>
       </c>
-      <c r="B167" s="3" t="s">
+    </row>
+    <row r="112">
+      <c r="A112" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="168" ht="15.75" customHeight="1">
-      <c r="A168" s="3" t="s">
+      <c r="B112" t="s">
         <v>334</v>
       </c>
-      <c r="B168" s="3" t="s">
+      <c r="C112" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="169" ht="15.75" customHeight="1">
-      <c r="A169" s="3" t="s">
+    <row r="113">
+      <c r="A113" t="s">
         <v>336</v>
       </c>
-      <c r="B169" s="3" t="s">
+      <c r="B113" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="170" ht="15.75" customHeight="1">
-      <c r="A170" s="3" t="s">
+      <c r="C113" t="s">
         <v>338</v>
       </c>
-      <c r="B170" s="3" t="s">
+    </row>
+    <row r="114">
+      <c r="A114" t="s">
         <v>339</v>
       </c>
-    </row>
-    <row r="171" ht="15.75" customHeight="1">
-      <c r="A171" s="3" t="s">
+      <c r="B114" t="s">
         <v>340</v>
       </c>
-      <c r="B171" s="3" t="s">
+      <c r="C114" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="172" ht="15.75" customHeight="1">
-      <c r="A172" s="3" t="s">
+    <row r="115">
+      <c r="A115" t="s">
         <v>342</v>
       </c>
-      <c r="B172" s="3" t="s">
+      <c r="B115" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="173" ht="15.75" customHeight="1">
-      <c r="A173" s="3" t="s">
+      <c r="C115" t="s">
         <v>344</v>
       </c>
-      <c r="B173" s="3" t="s">
+    </row>
+    <row r="116">
+      <c r="A116" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="174" ht="15.75" customHeight="1">
-      <c r="A174" s="3" t="s">
+      <c r="B116" t="s">
         <v>346</v>
       </c>
-      <c r="B174" s="3" t="s">
+      <c r="C116" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="175" ht="15.75" customHeight="1">
-      <c r="A175" s="3" t="s">
+    <row r="117">
+      <c r="A117" t="s">
         <v>348</v>
       </c>
-      <c r="B175" s="3" t="s">
+      <c r="B117" t="s">
         <v>349</v>
       </c>
-    </row>
-    <row r="176" ht="15.75" customHeight="1">
-      <c r="A176" s="3" t="s">
+      <c r="C117" t="s">
         <v>350</v>
       </c>
-      <c r="B176" s="3" t="s">
+    </row>
+    <row r="118">
+      <c r="A118" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="177" ht="15.75" customHeight="1">
-      <c r="A177" s="3" t="s">
+      <c r="B118" t="s">
         <v>352</v>
       </c>
-      <c r="B177" s="3" t="s">
+      <c r="C118" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="178" ht="15.75" customHeight="1">
-      <c r="A178" s="3" t="s">
+    <row r="119">
+      <c r="A119" t="s">
         <v>354</v>
       </c>
-      <c r="B178" s="3" t="s">
+      <c r="B119" t="s">
         <v>355</v>
       </c>
-    </row>
-    <row r="179" ht="15.75" customHeight="1">
-      <c r="A179" s="3" t="s">
+      <c r="C119" t="s">
         <v>356</v>
       </c>
-      <c r="B179" s="3" t="s">
+    </row>
+    <row r="120">
+      <c r="A120" t="s">
         <v>357</v>
       </c>
-    </row>
-    <row r="180" ht="15.75" customHeight="1">
-      <c r="A180" s="3" t="s">
+      <c r="B120" t="s">
         <v>358</v>
       </c>
-      <c r="B180" s="3" t="s">
+      <c r="C120" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="181" ht="15.75" customHeight="1">
-      <c r="A181" s="3" t="s">
+    <row r="121">
+      <c r="A121" t="s">
         <v>360</v>
       </c>
-      <c r="B181" s="3" t="s">
+      <c r="B121" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="182" ht="15.75" customHeight="1">
-      <c r="A182" s="3" t="s">
+      <c r="C121" t="s">
         <v>362</v>
       </c>
-      <c r="B182" s="3" t="s">
+    </row>
+    <row r="122">
+      <c r="A122" t="s">
         <v>363</v>
       </c>
-    </row>
-    <row r="183" ht="15.75" customHeight="1"/>
+      <c r="B122" t="s">
+        <v>364</v>
+      </c>
+      <c r="C122" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="s">
+        <v>366</v>
+      </c>
+      <c r="B123" t="s">
+        <v>367</v>
+      </c>
+      <c r="C123" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="s">
+        <v>369</v>
+      </c>
+      <c r="B124" t="s">
+        <v>370</v>
+      </c>
+      <c r="C124" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="s">
+        <v>372</v>
+      </c>
+      <c r="B125" t="s">
+        <v>373</v>
+      </c>
+      <c r="C125" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="s">
+        <v>375</v>
+      </c>
+      <c r="B126" t="s">
+        <v>376</v>
+      </c>
+      <c r="C126" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="s">
+        <v>378</v>
+      </c>
+      <c r="B127" t="s">
+        <v>379</v>
+      </c>
+      <c r="C127" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="s">
+        <v>381</v>
+      </c>
+      <c r="B128" t="s">
+        <v>382</v>
+      </c>
+      <c r="C128" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="s">
+        <v>384</v>
+      </c>
+      <c r="B129" t="s">
+        <v>385</v>
+      </c>
+      <c r="C129" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="s">
+        <v>387</v>
+      </c>
+      <c r="B130" t="s">
+        <v>388</v>
+      </c>
+      <c r="C130" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="s">
+        <v>390</v>
+      </c>
+      <c r="B131" t="s">
+        <v>391</v>
+      </c>
+      <c r="C131" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="s">
+        <v>393</v>
+      </c>
+      <c r="B132" t="s">
+        <v>394</v>
+      </c>
+      <c r="C132" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="s">
+        <v>396</v>
+      </c>
+      <c r="B133" t="s">
+        <v>397</v>
+      </c>
+      <c r="C133" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="s">
+        <v>399</v>
+      </c>
+      <c r="B134" t="s">
+        <v>400</v>
+      </c>
+      <c r="C134" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="s">
+        <v>402</v>
+      </c>
+      <c r="B135" t="s">
+        <v>403</v>
+      </c>
+      <c r="C135" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="s">
+        <v>405</v>
+      </c>
+      <c r="B136" t="s">
+        <v>406</v>
+      </c>
+      <c r="C136" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="s">
+        <v>408</v>
+      </c>
+      <c r="B137" t="s">
+        <v>409</v>
+      </c>
+      <c r="C137" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="s">
+        <v>411</v>
+      </c>
+      <c r="B138" t="s">
+        <v>412</v>
+      </c>
+      <c r="C138" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="s">
+        <v>414</v>
+      </c>
+      <c r="B139" t="s">
+        <v>415</v>
+      </c>
+      <c r="C139" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="s">
+        <v>417</v>
+      </c>
+      <c r="B140" t="s">
+        <v>418</v>
+      </c>
+      <c r="C140" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="s">
+        <v>420</v>
+      </c>
+      <c r="B141" t="s">
+        <v>421</v>
+      </c>
+      <c r="C141" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="s">
+        <v>423</v>
+      </c>
+      <c r="B142" t="s">
+        <v>424</v>
+      </c>
+      <c r="C142" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="s">
+        <v>426</v>
+      </c>
+      <c r="B143" t="s">
+        <v>427</v>
+      </c>
+      <c r="C143" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="s">
+        <v>429</v>
+      </c>
+      <c r="B144" t="s">
+        <v>430</v>
+      </c>
+      <c r="C144" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="s">
+        <v>432</v>
+      </c>
+      <c r="B145" t="s">
+        <v>433</v>
+      </c>
+      <c r="C145" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="s">
+        <v>435</v>
+      </c>
+      <c r="B146" t="s">
+        <v>436</v>
+      </c>
+      <c r="C146" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="s">
+        <v>438</v>
+      </c>
+      <c r="B147" t="s">
+        <v>439</v>
+      </c>
+      <c r="C147" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="s">
+        <v>441</v>
+      </c>
+      <c r="B148" t="s">
+        <v>442</v>
+      </c>
+      <c r="C148" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="s">
+        <v>444</v>
+      </c>
+      <c r="B149" t="s">
+        <v>445</v>
+      </c>
+      <c r="C149" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="s">
+        <v>447</v>
+      </c>
+      <c r="B150" t="s">
+        <v>448</v>
+      </c>
+      <c r="C150" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="s">
+        <v>450</v>
+      </c>
+      <c r="B151" t="s">
+        <v>451</v>
+      </c>
+      <c r="C151" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="s">
+        <v>453</v>
+      </c>
+      <c r="B152" t="s">
+        <v>454</v>
+      </c>
+      <c r="C152" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="s">
+        <v>456</v>
+      </c>
+      <c r="B153" t="s">
+        <v>457</v>
+      </c>
+      <c r="C153" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="s">
+        <v>459</v>
+      </c>
+      <c r="B154" t="s">
+        <v>460</v>
+      </c>
+      <c r="C154" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="s">
+        <v>462</v>
+      </c>
+      <c r="B155" t="s">
+        <v>463</v>
+      </c>
+      <c r="C155" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="s">
+        <v>465</v>
+      </c>
+      <c r="B156" t="s">
+        <v>466</v>
+      </c>
+      <c r="C156" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="s">
+        <v>468</v>
+      </c>
+      <c r="B157" t="s">
+        <v>469</v>
+      </c>
+      <c r="C157" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="s">
+        <v>471</v>
+      </c>
+      <c r="B158" t="s">
+        <v>472</v>
+      </c>
+      <c r="C158" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="s">
+        <v>474</v>
+      </c>
+      <c r="B159" t="s">
+        <v>475</v>
+      </c>
+      <c r="C159" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="s">
+        <v>477</v>
+      </c>
+      <c r="B160" t="s">
+        <v>478</v>
+      </c>
+      <c r="C160" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="s">
+        <v>480</v>
+      </c>
+      <c r="B161" t="s">
+        <v>481</v>
+      </c>
+      <c r="C161" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="s">
+        <v>483</v>
+      </c>
+      <c r="B162" t="s">
+        <v>484</v>
+      </c>
+      <c r="C162" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="s">
+        <v>486</v>
+      </c>
+      <c r="B163" t="s">
+        <v>487</v>
+      </c>
+      <c r="C163" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="s">
+        <v>489</v>
+      </c>
+      <c r="B164" t="s">
+        <v>490</v>
+      </c>
+      <c r="C164" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="s">
+        <v>492</v>
+      </c>
+      <c r="B165" t="s">
+        <v>493</v>
+      </c>
+      <c r="C165" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="s">
+        <v>495</v>
+      </c>
+      <c r="B166" t="s">
+        <v>496</v>
+      </c>
+      <c r="C166" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="s">
+        <v>498</v>
+      </c>
+      <c r="B167" t="s">
+        <v>499</v>
+      </c>
+      <c r="C167" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="s">
+        <v>501</v>
+      </c>
+      <c r="B168" t="s">
+        <v>502</v>
+      </c>
+      <c r="C168" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="s">
+        <v>504</v>
+      </c>
+      <c r="B169" t="s">
+        <v>505</v>
+      </c>
+      <c r="C169" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="s">
+        <v>507</v>
+      </c>
+      <c r="B170" t="s">
+        <v>508</v>
+      </c>
+      <c r="C170" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="s">
+        <v>510</v>
+      </c>
+      <c r="B171" t="s">
+        <v>511</v>
+      </c>
+      <c r="C171" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="s">
+        <v>513</v>
+      </c>
+      <c r="B172" t="s">
+        <v>514</v>
+      </c>
+      <c r="C172" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="s">
+        <v>516</v>
+      </c>
+      <c r="B173" t="s">
+        <v>517</v>
+      </c>
+      <c r="C173" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="s">
+        <v>519</v>
+      </c>
+      <c r="B174" t="s">
+        <v>520</v>
+      </c>
+      <c r="C174" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="s">
+        <v>522</v>
+      </c>
+      <c r="B175" t="s">
+        <v>523</v>
+      </c>
+      <c r="C175" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="s">
+        <v>525</v>
+      </c>
+      <c r="B176" t="s">
+        <v>526</v>
+      </c>
+      <c r="C176" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="s">
+        <v>528</v>
+      </c>
+      <c r="B177" t="s">
+        <v>529</v>
+      </c>
+      <c r="C177" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="s">
+        <v>531</v>
+      </c>
+      <c r="B178" t="s">
+        <v>532</v>
+      </c>
+      <c r="C178" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="s">
+        <v>534</v>
+      </c>
+      <c r="B179" t="s">
+        <v>535</v>
+      </c>
+      <c r="C179" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="s">
+        <v>537</v>
+      </c>
+      <c r="B180" t="s">
+        <v>538</v>
+      </c>
+      <c r="C180" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="s">
+        <v>540</v>
+      </c>
+      <c r="B181" t="s">
+        <v>541</v>
+      </c>
+      <c r="C181" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="s">
+        <v>543</v>
+      </c>
+      <c r="B182" t="s">
+        <v>544</v>
+      </c>
+      <c r="C182" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="183"/>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>